<commit_message>
docs: sladění rozhodnutí o větvení a úpravách plánu
- Otázky na klienta: odebrán návrh lineárního plánu pro MVP (větvení zůstává v MVP).
- Otázky na klienta: úpravy plánu předpokládáme u psovoda i trenéra, k potvrzení s PO.
- Feature breakdown F-16: role „Psovod, trenér“, otevřená otázka změněna na potvrzení předpokladu.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature breakdown" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epicy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Návod" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Feature breakdown" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Epicy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Návod" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature breakdown'!$A$4:$I$60</definedName>
@@ -746,7 +746,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Potřebuje to MVP, nebo stačí jeden pes?</t>
+          <t>Rozhodnuto: v MVP plně podporováno (přepínání psů a barevné proužky v kalendáři). Bezplatný psovod může mít více psů pod trenérem.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1180,12 +1180,12 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Trenér po reakci na odeslaný trénink upraví plán v Tvorbě tréninku.</t>
+          <t>Psovod i trenér mohou upravit plán v Tvorbě tréninku. Trenér navíc po reakci na odeslaný trénink plán upraví.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Má plán upravovat i psovod? (otázka 2)</t>
+          <t>Předpoklad: plán upravují oba (psovod i trenér). Potvrdit s PO. (otázka 2)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Vlastní úložiště videí je drahé, v MVP ho nestavíme (viz F-25, otázka 4).</t>
+          <t>Vlastní úložiště videí je drahé, v MVP ho nestavíme (viz F-25, otázka 6).</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>Stačí web použitelný na mobilu, nebo je potřeba nativní aplikace?</t>
+          <t>Rozhodnuto: responzivní webová aplikace (optimalizovaná pro mobil / PWA). Nativní aplikace v App Store / Google Play mimo rozsah pilotu.</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: zapracování rozhovoru s trenérkou a FB1
- plán úprav (plan-uprav-po-fb1.md) se zjištěními z rozhovoru a rozhodnutími PO
- Lean Canvas 1.3 (.md i .docx): problém, alternativy, UVP, segmenty, metriky, náklady
- feature breakdown: stavy podle upraveného plánu a FB1, zdroj Rozhovor, nové F-44 až F-46, řádky seřazené podle epiců
- sitemapa (.md i .svg): pojmy cíl a záznam, přesun/přeskočení, záznam tréninku s vláknem, stav wireframů
- výsledky rozhovoru: doplněny H7, H8 a mezery
- otázky: zodpovězené z FB1 označeny, nové v otazky-fb2.md
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Feature breakdown" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Epicy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Návod" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature breakdown" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epicy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Návod" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature breakdown'!$A$4:$I$60</definedName>
@@ -434,7 +434,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tým 5 · nástřel na hackathon 9. 10. 2026, sladěný s wireframem ve Figmě, vše ve stavu „Navrženo“ k projednání s PO. Čísla otázek v závorce odkazují na otazky-na-klienta.md. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
+          <t>Tým 5 · aktualizace 9. 10. 2026 po rozhovoru s trenérkou a FB1. „Odsouhlaseno“ = rozhodl upravený plán nebo PO ve FB1, „Navrženo“ = k projednání. „FB2, otázka N“ odkazuje na otazky-fb2.md. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
         </is>
       </c>
     </row>
@@ -518,17 +518,17 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto: trenér je placený účet a zve klienty. Může psovod aplikaci používat i bez trenéra? (otázka 2, 10)</t>
+          <t>Rozhodnuto (UP): platí trenér, psovod se registruje přes jeho pozvánku a má aplikaci zdarma.</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
@@ -654,14 +654,10 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Jaké další údaje jsou potřeba (věk, zdravotní omezení)?</t>
-        </is>
-      </c>
+      <c r="H8" s="5" t="n"/>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
@@ -704,7 +700,7 @@
       <c r="H9" s="5" t="n"/>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
@@ -746,12 +742,12 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto: v MVP plně podporováno (přepínání psů a barevné proužky v kalendáři). Bezplatný psovod může mít více psů pod trenérem.</t>
+          <t>Rozhodnuto (UP): více psů na účtu psovoda, i pod trenérem zdarma.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
@@ -801,22 +797,22 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>F-08</t>
+          <t>F-45</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Sdílení s trenérem</t>
+          <t>Pes a disciplíny</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Trenér pozve klienta</t>
+          <t>Vlastní psi trenéra</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Trenér pošle klientovi pozvánku e-mailem nebo mu předá kód (třeba na lekci). Aplikaci platí trenér, proto zve on.</t>
+          <t>Trenér vede v aplikaci i své psy místo papírového deníku (respondentka má 3 psy a deník na každého psa a sport).</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -826,17 +822,17 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Zve trenér člověka, nebo konkrétního psa? Co když klient už účet má? (otázka 8)</t>
+          <t>Chce to trenér? (FB2, otázka 6)</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -848,7 +844,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>F-09</t>
+          <t>F-08</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -858,17 +854,17 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Přijetí pozvánky („Mám pozvánku“)</t>
+          <t>Trenér pozve klienta</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Klient na úvodní obrazovce zvolí „Mám pozvánku“, zadá kód nebo otevře odkaz, zaregistruje se a propojí se s trenérem.</t>
+          <t>Trenér pošle klientovi pozvánku e-mailem nebo mu předá kód (třeba na lekci). Aplikaci platí trenér, proto zve on.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -878,24 +874,24 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Jak dlouho kód platí? (otázka 8)</t>
+          <t>Rozhodnuto (UP): zve trenér e-mailem nebo kódem. Trenér zve člověka, klient po přijetí vybere nebo založí psa.</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>F-10</t>
+          <t>F-09</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -905,17 +901,17 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Odebrání přístupu</t>
+          <t>Přijetí pozvánky („Mám pozvánku“)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Trenér nebo psovod ukončí spolupráci, trenér psa přestane vidět.</t>
+          <t>Klient na úvodní obrazovce zvolí „Mám pozvánku“, zadá kód nebo otevře odkaz, zaregistruje se a propojí se s trenérem.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -925,20 +921,24 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Kód platí 7 dní (návrh týmu).</t>
+        </is>
+      </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>F-11</t>
+          <t>F-10</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -948,22 +948,22 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Psovod pozve trenéra</t>
+          <t>Odebrání přístupu</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Obrácený směr: psovod, který už trenéra má, ho pozve do aplikace.</t>
+          <t>Trenér nebo psovod ukončí spolupráci, trenér psa přestane vidět.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -971,7 +971,7 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr"/>
+      <c r="H15" s="5" t="n"/>
       <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -981,44 +981,40 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>F-12</t>
+          <t>F-11</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku</t>
+          <t>Sdílení s trenérem</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku pro psa</t>
+          <t>Psovod pozve trenéra</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Trenér založí pro psa klienta plán v disciplíně, např. „Trénink pro Rexe“ (obrazovka Tvorba tréninku).</t>
+          <t>Obrácený směr: psovod, který už trenéra má, ho pozve do aplikace.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Chcete u plánu i cíl (např. 5 km pod 5 min/km)? (otázka 4)</t>
-        </is>
-      </c>
+          <t>Předpoklad týmu</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="n"/>
       <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1028,7 +1024,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>F-13</t>
+          <t>F-12</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1038,12 +1034,12 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Cviky a sekvence cviků</t>
+          <t>Cíl a plán tréninku</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Plán se skládá z bloků „Jednotlivý cvik“ (např. Běh v plném tahu 400 m) a „Sekvence cviků“ (několik cviků vždy po sobě). Blok jde přidat (+), upravit, smazat (koš) nebo vložit jako mezikrok.</t>
+          <t>Trenér založí pro psa klienta cíl v disciplíně, dlouhodobý (spolehlivá chůze u nohy) i drobný trik (pac). Plán začíná principem: čeho docílit a na co si dát pozor. Trenérka v rozhovoru zadává nejdřív princip, pak cviky.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1061,17 +1057,21 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Rozhodnuto (PO, FB1): plán musí unést dlouhodobé cíle i drobné triky.</t>
+        </is>
+      </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>F-14</t>
+          <t>F-13</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1081,12 +1081,12 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Posun, návrat a přeskočení</t>
+          <t>Cviky a sekvence cviků</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Je vidět, na kterém cviku pes je. Když nejde, vrátí se o krok; když to umí, cvik se přeskočí.</t>
+          <t>Plán se skládá z bloků „Jednotlivý cvik“ a „Sekvence cviků“. Každý cvik má instrukci a kritérium zvládnutí („sedí, i když kolem letí míčky“), aby klient doma věděl, co přesně cvičit. Blok jde přidat, upravit, smazat nebo vložit jako mezikrok.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1101,12 +1101,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Posouvá se jen ručně, nebo i podle % úspěšnosti? (otázka 1)</t>
+          <t>Instrukce a kritérium u cviku jsou z rozhovoru (klienti si ústní zadání nezapamatují). Potvrdit na FB2.</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1118,7 +1118,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>F-15</t>
+          <t>F-14</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1128,12 +1128,12 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Rozvětvení cesty</t>
+          <t>Posun, návrat a přeskočení</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Cesta se rozdělí na dvě větve, které se trénují souběžně, a později se mohou znovu spojit (tak to kreslí wireframe).</t>
+          <t>Je vidět, na kterém cviku pes je. Když nejde („tunel“, opakuje stejnou chybu), vrátí se o krok; když to umí, cvik se přeskočí. O posunu rozhoduje člověk podle chování psa.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1151,21 +1151,17 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>Větví se plán na několik týdnů, nebo jeden trénink? Trénují se obě větve, nebo se jedna vybere? Příklad se Zoe. (otázka 1)</t>
-        </is>
-      </c>
+      <c r="H19" s="5" t="n"/>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>F-16</t>
+          <t>F-15</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1175,17 +1171,17 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Úpravy plánu podle výsledků</t>
+          <t>Rozvětvení cesty</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Psovod i trenér mohou upravit plán v Tvorbě tréninku. Trenér navíc po reakci na odeslaný trénink plán upraví.</t>
+          <t>Cesta se rozvětví. Pro MVP v jednoduché podobě: krok, který pes nechápe, se rozdělí na dílčí kroky a po jejich zvládnutí se cesta vrací do hlavní linie („nejdřív kousky, pak celek“). Datový model nepřekombinovat (PO, FB1).</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1200,19 +1196,19 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad: plán upravují oba (psovod i trenér). Potvrdit s PO. (otázka 2)</t>
+          <t>Podobu ukázat na FB2 (otázka 1).</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>F-17</t>
+          <t>F-16</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1222,17 +1218,17 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Dokončení a archiv plánu</t>
+          <t>Úpravy plánu podle výsledků</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Dokončený nebo opuštěný plán zmizí z aktivních, ale zůstane v historii.</t>
+          <t>Psovod i trenér mohou upravit plán v Tvorbě tréninku. Trenér navíc po reakci na odeslaný trénink plán upraví.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1242,20 +1238,24 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Rozhodnuto (UP): plán upravují psovod i trenér.</t>
+        </is>
+      </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>F-18</t>
+          <t>F-17</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Kopie plánu / šablona trenéra</t>
+          <t>Dokončení a archiv plánu</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Trenér zkopíruje osvědčený plán k dalšímu psovi.</t>
+          <t>Dokončený nebo opuštěný plán zmizí z aktivních, ale zůstane v historii.</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1298,40 +1298,44 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>F-19</t>
+          <t>F-18</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Týdenní rozvrh</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Týdenní kalendář</t>
+          <t>Kopie plánu / šablona trenéra</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Aktuální týden po dnech, tréninky všech psů najednou, barevně podle psa. Po kliknutí na den karta tréninku se seznamem cviků.</t>
+          <t>Trenér zkopíruje osvědčený plán k dalšímu psovi.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="n"/>
+          <t>Předpoklad týmu</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Dávají trenéři podobné plány více klientům? (FB2, otázka 7)</t>
+        </is>
+      </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1341,7 +1345,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>F-20</t>
+          <t>F-19</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1351,17 +1355,17 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Naplánování tréninku na den</t>
+          <t>Týdenní kalendář</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Trenér po uložení tréninku vybere dny v týdnu a období (od–do). Trénink se objeví klientovi v Týdnu.</t>
+          <t>Aktuální týden po dnech, tréninky všech psů najednou, barevně podle psa. Po kliknutí na den karta tréninku se seznamem cviků.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1374,21 +1378,17 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Vybere dny trenér, nebo má aplikace trénink rozvrhnout sama („vygenerovaný popis“ ve wireframu)? (otázka 5)</t>
-        </is>
-      </c>
+      <c r="H24" s="5" t="n"/>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>F-21</t>
+          <t>F-20</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1398,17 +1398,17 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Přesun mezi dny</t>
+          <t>Naplánování tréninku na den</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Naplánovaný trénink jde přesunout na jiný den.</t>
+          <t>Tréninky se zařadí do dnů v týdnu a období (od–do). Rozvrh se zobrazuje v týdnech a dnech jako v aplikaci Runna.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -1421,7 +1421,11 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H25" s="5" t="n"/>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Kdo zařazuje tréninky do dnů, trenér, nebo psovod? (FB2, otázka 2)</t>
+        </is>
+      </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1431,7 +1435,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>F-22</t>
+          <t>F-21</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1441,12 +1445,12 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Přepínání týdnů</t>
+          <t>Přesunout, nebo přeskočit trénink</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Zpět (co se odcvičilo) i dopředu (plánování).</t>
+          <t>Když trénink v daný den neproběhne, psovod ho jedním krokem přesune na jiný den či týden, nebo ho přeskočí, aby nevznikala lavina nedodělků (vzor Runna).</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1461,20 +1465,24 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Co se stane s přeskočeným cvikem v plánu a vidí to trenér? (FB2, otázka 4)</t>
+        </is>
+      </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>F-23</t>
+          <t>F-22</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1484,12 +1492,12 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Neodcvičené tréninky a zanedbané disciplíny</t>
+          <t>Přepínání týdnů</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Upozornění, co se neodcvičilo nebo která disciplína tento týden nemá trénink.</t>
+          <t>Zpět (co se odcvičilo) i dopředu (plánování).</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1499,7 +1507,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -1507,11 +1515,7 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>Co se má stát s neodcvičeným tréninkem?</t>
-        </is>
-      </c>
+      <c r="H27" s="5" t="n"/>
       <c r="I27" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1521,22 +1525,22 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>F-24</t>
+          <t>F-23</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Týdenní rozvrh</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Odeslání tréninku</t>
+          <t>Zanedbané disciplíny</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Na obrazovce „Konec“ psovod napíše komentář a odešle trénink trenérovi — rychle, z mobilu.</t>
+          <t>Upozornění, že některá disciplína tento týden nemá trénink. Neodcvičené tréninky řeší F-21.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1546,17 +1550,17 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Má psovod zadávat i % úspěšnosti? Za každý cvik, nebo za celý trénink? (otázka 3)</t>
+          <t>Více disciplín trenérce práci navíc nedělá (H1 oslabena).</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -1568,7 +1572,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>F-25</t>
+          <t>F-43</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1578,12 +1582,12 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Video z tréninku</t>
+          <t>Průchod tréninkem</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Na obrazovce „Konec“ psovod tlačítkem „Nahrát video“ přiloží video z tréninku, takže už neleží odpojené v galerii.</t>
+          <t>Psovod otevře dnešní trénink a prochází cviky jeden po druhém („Aktuální cvik 3/20“), na konci přejde na obrazovku „Konec“.</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1598,12 +1602,12 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Stačí v MVP odkaz (YouTube, Disk), nebo nahrání souboru (F-28)? (otázka 6)</t>
+          <t>Šipky = další cvik v dnešním tréninku. Každý cvik ukazuje instrukci a kritérium (F-13).</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -1615,7 +1619,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>F-26</t>
+          <t>F-24</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1625,17 +1629,17 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Historie tréninků psa</t>
+          <t>Odeslání tréninku</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Na detailu psa jsou „Aktivity“: odcvičené tréninky po dnech se záznamy, jde porovnat, co fungovalo.</t>
+          <t>Na obrazovce „Konec“ psovod zadá % úspěšnosti, rychlé hodnocení (soustředění, opakované chyby) a poznámku a odešle trénink trenérovi. Rychle, z mobilu.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -1648,7 +1652,11 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H30" s="5" t="n"/>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Za cvik, nebo za celý trénink? Jak má psovod % určit? Trenérka měří úspěch kvalitativně (H5). (FB2, otázka 3)</t>
+        </is>
+      </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1658,7 +1666,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>F-27</t>
+          <t>F-25</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1668,44 +1676,44 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Graf vývoje úspěšnosti</t>
+          <t>Video z tréninku</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Vývoj % v čase u psa nebo plánu.</t>
+          <t>Na obrazovce „Konec“ psovod vloží odkaz na video z tréninku (YouTube unlisted, cloud), takže video už neleží odpojené v galerii.</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Jen pokud se bude zadávat % úspěšnosti (otázka 3).</t>
+          <t>Jak klientům vložení odkazu usnadnit? (FB2, otázka 11)</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>F-28</t>
+          <t>F-44</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1715,12 +1723,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Nahrávání videí na náš server</t>
+          <t>Kontext k záznamu</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Vlastní úložiště videí je drahé, v MVP ho nestavíme (viz F-25, otázka 6).</t>
+          <t>Psovod u záznamu volitelně vyplní okolnosti (jak pes spal, prostředí, jestli se chyba opakuje), na které se trenérka jinak doptává.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1730,12 +1738,12 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Mimo rozsah</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H32" s="5" t="n"/>
@@ -1748,7 +1756,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>F-29</t>
+          <t>F-26</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1758,22 +1766,22 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Napojení na Stravu</t>
+          <t>Historie tréninků psa</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Import canicrossových běhů z běžeckých aplikací.</t>
+          <t>Na detailu psa jsou „Aktivity“: odcvičené tréninky po dnech s videi a odpověďmi trenéra. Hodnota hlavně pro psovoda, který se k videím a zpětné vazbě vrací (trenérka ne).</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Mimo rozsah</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -1791,22 +1799,22 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>F-30</t>
+          <t>F-27</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Zpětná vazba</t>
+          <t>Záznam tréninku</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Komentáře k tréninku</t>
+          <t>Graf vývoje úspěšnosti</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Psovod pošle s tréninkem komentář, trenér mu odpoví ve vlákně a reaguje na video. Nahrazuje WhatsApp.</t>
+          <t>Vývoj % v čase u psa nebo plánu.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1816,17 +1824,17 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Kde psovod odpověď trenéra uvidí? (otázka 9)</t>
+          <t>Úspěch se v praxi číslem neměří (H5 podpořena).</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -1838,32 +1846,32 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>F-31</t>
+          <t>F-28</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Zpětná vazba</t>
+          <t>Záznam tréninku</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Seznam klientů</t>
+          <t>Nahrávání videí na náš server</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Trenér vidí své klienty (jméno, e-mail) a přes ně jejich psy, plány a odcvičené tréninky.</t>
+          <t>Vlastní úložiště videí je drahé, v MVP ho nestavíme (viz F-25, otázka 6).</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -1874,44 +1882,44 @@
       <c r="H35" s="5" t="n"/>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>F-32</t>
+          <t>F-29</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Zpětná vazba</t>
+          <t>Záznam tréninku</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Čeká na reakci</t>
+          <t>Napojení na Stravu</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>U klienta svítí štítek „čeká na reakci“, dokud trenér nezareaguje na jeho nové záznamy.</t>
+          <t>Import canicrossových běhů z běžeckých aplikací.</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H36" s="5" t="n"/>
@@ -1924,7 +1932,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>F-33</t>
+          <t>F-30</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1934,12 +1942,12 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Upozornění</t>
+          <t>Komentáře k tréninku</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Psovod nebo trenér se dozví o novém komentáři, záznamu nebo změně plánu.</t>
+          <t>Psovod pošle s tréninkem komentář, trenér mu odpoví ve vlákně pod konkrétním tréninkem a reaguje na video. Vlákno unese dialog i doptávání (jak pes spal, jestli se chyba opakuje). Nahrazuje WhatsApp.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -1949,54 +1957,50 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>E-mail, nebo stačí upozornění v aplikaci?</t>
-        </is>
-      </c>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="n"/>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>F-34</t>
+          <t>F-31</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Tržiště a platby</t>
+          <t>Zpětná vazba</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Prodej a nákup plánů, hodnocení</t>
+          <t>Seznam klientů</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Veřejné tržiště plánů z původního briefu.</t>
+          <t>Trenér vidí své klienty (jméno, e-mail) a přes ně jejich psy, plány a odcvičené tréninky.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Mimo rozsah</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -2004,32 +2008,36 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H38" s="5" t="n"/>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>Potvrzeno (PO, FB1): horní přehled svěřenců odpovídá pohledu trenéra.</t>
+        </is>
+      </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>F-35</t>
+          <t>F-32</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Tržiště a platby</t>
+          <t>Zpětná vazba</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Předplatné a platby</t>
+          <t>Čeká na reakci</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Budoucí předplatné pro trenéry, tento semestr bez plateb.</t>
+          <t>Fronta dotazů a záznamů od klientů, na které trenér ještě neodpověděl. Slouží jako pomocník, ne kontrola plnění: trenérka od klientů nic nevyžaduje a pokrok pozná na další lekci.</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2039,12 +2047,12 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Mimo rozsah</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H39" s="5" t="n"/>
@@ -2057,27 +2065,27 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>F-36</t>
+          <t>F-33</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Technický základ</t>
+          <t>Zpětná vazba</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Staging a CI/CD</t>
+          <t>Štítek „nová odpověď“</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Každá změna se otestuje a nasadí na staging, kde ji PO uvidí dřív než uživatelé.</t>
+          <t>Psovod v Týdnu a u tréninku vidí, že mu trenér odpověděl; trenér vidí nové záznamy. Bez toho psovod odpověď nenajde.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
@@ -2087,14 +2095,10 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="H40" s="5" t="inlineStr">
-        <is>
-          <t>Kdo bude mít přístup na staging?</t>
-        </is>
-      </c>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="n"/>
       <c r="I40" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -2104,40 +2108,44 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>F-37</t>
+          <t>F-46</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Technický základ</t>
+          <t>Zpětná vazba</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Automatické testy</t>
+          <t>E-mailová upozornění</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Hlavní obrana proti chybám od agenta, hlavně v logice nelineárního plánu.</t>
+          <t>Psovod nebo trenér dostane e-mail o nové odpovědi, záznamu nebo změně plánu.</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="n"/>
+          <t>Předpoklad týmu</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Stačí upozornění v aplikaci, nebo je potřeba i e-mail? (FB2, otázka 5)</t>
+        </is>
+      </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -2147,93 +2155,93 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>F-38</t>
+          <t>F-34</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Technický základ</t>
+          <t>Tržiště a platby</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Oprávnění</t>
+          <t>Prodej a nákup plánů, hodnocení</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Kdo vidí a upravuje psa, plán, záznamy a komentáře (psovod, trenér, cizí).</t>
+          <t>Veřejné tržiště plánů z původního briefu.</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H42" s="5" t="n"/>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>F-39</t>
+          <t>F-35</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Technický základ</t>
+          <t>Tržiště a platby</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Osobní údaje a smazání účtu</t>
+          <t>Předplatné a platby</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Souhlas se zpracováním, smazání účtu včetně dat.</t>
+          <t>Budoucí předplatné pro trenéry, tento semestr bez plateb.</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H43" s="5" t="n"/>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>F-40</t>
+          <t>F-36</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -2243,17 +2251,17 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Použitelnost na mobilu</t>
+          <t>Staging a CI/CD</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Psovod zapisuje venku po tréninku, aplikace musí fungovat na telefonu.</t>
+          <t>Každá změna se otestuje a nasadí na staging, kde ji PO uvidí dřív než uživatelé.</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -2263,12 +2271,12 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto: responzivní webová aplikace (optimalizovaná pro mobil / PWA). Nativní aplikace v App Store / Google Play mimo rozsah pilotu.</t>
+          <t>Kdo bude mít přístup na staging?</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
@@ -2280,7 +2288,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>F-41</t>
+          <t>F-37</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -2290,12 +2298,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Zálohy dat</t>
+          <t>Automatické testy</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Pravidelná záloha databáze, aby historie tréninků nezmizela.</t>
+          <t>Hlavní obrana proti chybám od agenta, hlavně v logice nelineárního plánu.</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2323,7 +2331,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>F-42</t>
+          <t>F-38</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -2333,12 +2341,12 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Monitoring a logy</t>
+          <t>Oprávnění</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>O chybě se dozvíme dřív než uživatel.</t>
+          <t>Kdo vidí a upravuje psa, plán, záznamy a komentáře (psovod, trenér, cizí).</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2348,7 +2356,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -2366,27 +2374,27 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>F-43</t>
+          <t>F-39</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Technický základ</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Průchod tréninkem</t>
+          <t>Osobní údaje a smazání účtu</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Psovod otevře dnešní trénink a prochází cviky jeden po druhém („Aktuální cvik 3/20“), na konci přejde na obrazovku „Konec“.</t>
+          <t>Souhlas se zpracováním, smazání účtu včetně dat.</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -2399,11 +2407,7 @@
           <t>Tým</t>
         </is>
       </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>Znamenají šipky další cvik v dnešním tréninku, nebo posun v plánu (F-14)?</t>
-        </is>
-      </c>
+      <c r="H47" s="5" t="n"/>
       <c r="I47" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -2411,37 +2415,137 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="n"/>
-      <c r="B48" s="5" t="n"/>
-      <c r="C48" s="5" t="n"/>
-      <c r="D48" s="5" t="n"/>
-      <c r="E48" s="5" t="n"/>
-      <c r="F48" s="5" t="n"/>
-      <c r="G48" s="5" t="n"/>
-      <c r="H48" s="5" t="n"/>
-      <c r="I48" s="5" t="n"/>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>F-40</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Technický základ</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Použitelnost na mobilu</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Psovod zapisuje venku po tréninku, aplikace musí fungovat na telefonu.</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Psovod, trenér</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>Rozhodnuto: responzivní webová aplikace (optimalizovaná pro mobil / PWA). Nativní aplikace v App Store / Google Play mimo rozsah pilotu.</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="n"/>
-      <c r="B49" s="5" t="n"/>
-      <c r="C49" s="5" t="n"/>
-      <c r="D49" s="5" t="n"/>
-      <c r="E49" s="5" t="n"/>
-      <c r="F49" s="5" t="n"/>
-      <c r="G49" s="5" t="n"/>
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>F-41</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Technický základ</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Zálohy dat</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Pravidelná záloha databáze, aby historie tréninků nezmizela.</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Tým</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Tým</t>
+        </is>
+      </c>
       <c r="H49" s="5" t="n"/>
-      <c r="I49" s="5" t="n"/>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Navrženo</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="n"/>
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="5" t="n"/>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>F-42</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Technický základ</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Monitoring a logy</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>O chybě se dozvíme dřív než uživatel.</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Tým</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Nice to have</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Tým</t>
+        </is>
+      </c>
       <c r="H50" s="5" t="n"/>
-      <c r="I50" s="5" t="n"/>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Navrženo</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>

</xml_diff>

<commit_message>
docs: propsání zjištění z rozhovoru do Lean Canvasu, breakdownu a otázek na FB 2
- zjištění z rozhovoru s trenérkou a vyhodnocení hypotéz
- Lean Canvas 1.3 (md i docx): jádro je zadání z lekce v telefonu klienta
- varianta B Lean Canvasu (psovod začíná s deníkem) k diskusi s PO
- feature breakdown: změny priorit (sloupec J), nové F-44 až F-47, MVP podbarvené
- otázky na FB 2 včetně toho, co zatím nevíme

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Návod" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature breakdown'!$A$4:$I$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature breakdown'!$A$4:$J$60</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -140,6 +140,16 @@
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2EFDA"/>
+          <bgColor rgb="00E2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -410,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -422,6 +432,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.7" customHeight="1">
@@ -434,7 +445,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tým 5 · nástřel na hackathon 9. 10. 2026, sladěný s wireframem ve Figmě, vše ve stavu „Navrženo“ k projednání s PO. Čísla otázek v závorce odkazují na otazky-na-klienta.md. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
+          <t>Tým 5 · verze po rozhovoru s uživatelkou (trenérkou) na hackathonu 9. 10. 2026. Vše ve stavu „Navrženo“ k projednání s PO ve FB 2. Sloupec J říká, co se po rozhovoru změnilo. Čísla otázek odkazují na otazky-fb2.md (zjištění v zjisteni-rozhovor-1.md). Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
         </is>
       </c>
     </row>
@@ -484,6 +495,11 @@
           <t>Stav</t>
         </is>
       </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Změna po rozhovoru (9. 10.)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -523,7 +539,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto: trenér je placený účet a zve klienty. Může psovod aplikaci používat i bez trenéra? (otázka 2, 10)</t>
+          <t>Rozhodnuto: trenér je placený účet a zve klienty. Může psovod aplikaci používat i bez trenéra? (FB2 otázka 10)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -531,6 +547,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -574,6 +591,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -617,6 +635,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -664,6 +683,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -701,12 +721,17 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H9" s="5" t="n"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>H1 oslabena: více disciplín trenérce práci navíc nedělá. Stačí disciplína jako štítek u zadání? (FB2 otázka 11)</t>
+        </is>
+      </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -754,6 +779,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -797,6 +823,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -844,6 +871,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -891,6 +919,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -934,6 +963,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -977,6 +1007,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -991,12 +1022,12 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku pro psa</t>
+          <t>Zadání z lekce pro klienta</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Trenér založí pro psa klienta plán v disciplíně, např. „Trénink pro Rexe“ (obrazovka Tvorba tréninku).</t>
+          <t>Trenér po lekci zapíše klientovi zadání pro psa: princip (čeho docílit), na co si dát pozor a konkrétní cviky. Dnes ho předává jen ústně, klienti si zapíšou jen část a doma nevědí, co cvičit.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1011,17 +1042,22 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Chcete u plánu i cíl (např. 5 km pod 5 min/km)? (otázka 4)</t>
+          <t>Kdo zadání píše a kolik času to smí trenéra stát? Trenérka má ~40 klientů měsíčně. (FB2 otázka 1, 2)</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Přeformulováno: z „plánu tréninku“ na zadání z lekce. Nové jádro MVP.</t>
         </is>
       </c>
     </row>
@@ -1038,12 +1074,12 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Cviky a sekvence cviků</t>
+          <t>Cviky, dílčí kroky a kritérium zvládnutí</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Plán se skládá z bloků „Jednotlivý cvik“ (např. Běh v plném tahu 400 m) a „Sekvence cviků“ (několik cviků vždy po sobě). Blok jde přidat (+), upravit, smazat (koš) nebo vložit jako mezikrok.</t>
+          <t>Cvik se skládá z dílčích kroků (chůze u nohy: pozice u nohy → pohyb u nohy → natočení zadkem). U cviku je kritérium zvládnutí, např. „sedí, i když kolem letí míčky“. Blok jde přidat, upravit nebo smazat, sekvence cviků zůstává.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1058,7 +1094,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H17" s="5" t="n"/>
@@ -1067,6 +1103,11 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Doplněny dílčí kroky a kritérium zvládnutí.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1081,12 +1122,12 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Posun, návrat a přeskočení</t>
+          <t>Návrat o krok a vložení mezikroku</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Je vidět, na kterém cviku pes je. Když nejde, vrátí se o krok; když to umí, cvik se přeskočí.</t>
+          <t>Je vidět, na kterém kroku pes je. Když opakuje stejnou chybu („tunel“) nebo je zbrklý, vrátí se o krok nebo se vloží mezikrok. Když to pes umí, krok se přeskočí. Posun je ruční.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1101,17 +1142,22 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Posouvá se jen ručně, nebo i podle % úspěšnosti? (otázka 1)</t>
+          <t>Rozhodnuto rozhovorem: posun ručně, ne podle % (pokrok se čte z chování psa).</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Doplněn mezikrok, posun jen ručně.</t>
         </is>
       </c>
     </row>
@@ -1143,22 +1189,27 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Větví se plán na několik týdnů, nebo jeden trénink? Trénují se obě větve, nebo se jedna vybere? Příklad se Zoe. (otázka 1)</t>
+          <t>Části cviku se nacvičí zvlášť a pak spojí, s přehledem ale trenérka problém nemá (H2 oslabena). Stačí v MVP dílčí kroky a mezikrok? (FB2 otázka 4)</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>MVP → Nice to have</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1251,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad: plán upravují oba (psovod i trenér). Potvrdit s PO. (otázka 2)</t>
+          <t>Upravují plán oba? Trenérka mění zadání na lekci, klienti trénují „po svým“. (FB2 otázka 2)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -1208,6 +1259,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1251,6 +1303,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1265,12 +1318,12 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Kopie plánu / šablona trenéra</t>
+          <t>Šablony cviků a zadání trenéra</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Trenér zkopíruje osvědčený plán k dalšímu psovi.</t>
+          <t>Trenér si uloží opakované cviky (sedni, chůze u nohy) i s kroky a kritérii a vloží je do zadání dalšímu klientovi. Bez toho je psaní zadání pro desítky klientů měsíčně práce navíc.</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1280,7 +1333,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1288,10 +1341,19 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H22" s="5" t="n"/>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Je zadání ze šablon dost rychlé, aby ho trenér psal po každé lekci? (FB2 otázka 2)</t>
+        </is>
+      </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Nice to have → MVP: podmínka, aby trenér zadání vůbec psal.</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1375,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Aktuální týden po dnech, tréninky všech psů najednou, barevně podle psa. Po kliknutí na den karta tréninku se seznamem cviků.</t>
+          <t>Aktuální týden po dnech, úkoly všech psů najednou, barevně podle psa. Po kliknutí na den karta tréninku se seznamem cviků.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1331,10 +1393,19 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H23" s="5" t="n"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Potřebuje klient, který chodí na lekci 1× za měsíc, kalendář, nebo stačí aktuální zadání u psa (F-47)? (FB2 otázka 6)</t>
+        </is>
+      </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Priorita beze změny, k ověření.</t>
         </is>
       </c>
     </row>
@@ -1351,17 +1422,17 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Naplánování tréninku na den</t>
+          <t>Rozvržení úkolů do týdne</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Trenér po uložení tréninku vybere dny v týdnu a období (od–do). Trénink se objeví klientovi v Týdnu.</t>
+          <t>Psovod si úkoly ze zadání sám rozvrhne do dnů v týdnu. Trenér dny nezadává: klienti chodí 1× za měsíc a trénují „po svým“.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1371,17 +1442,22 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Vybere dny trenér, nebo má aplikace trénink rozvrhnout sama („vygenerovaný popis“ ve wireframu)? (otázka 5)</t>
+          <t>Rozvrhuje psovod, nebo trenér? (FB2 otázka 6)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Role trenér → psovod.</t>
         </is>
       </c>
     </row>
@@ -1427,6 +1503,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1470,6 +1547,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1517,6 +1595,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1531,12 +1610,12 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Odeslání tréninku</t>
+          <t>Zápis tréninku a hodnocení slovy</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Na obrazovce „Konec“ psovod napíše komentář a odešle trénink trenérovi — rychle, z mobilu.</t>
+          <t>Po tréninku psovod zapíše, jak to šlo: Šlo / Částečně / Nešlo, co nefungovalo (opakuje stejnou chybu, zbrklý, nesoustředěný) a poznámku. Bez % úspěšnosti: trenérka pokrok čte z chování psa, ne z čísla.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1551,17 +1630,22 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Má psovod zadávat i % úspěšnosti? Za každý cvik, nebo za celý trénink? (otázka 3)</t>
+          <t>Má být zápis povinný? Trenérka zápisy od klientů nevyžaduje. (FB2 otázka 3)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Vypuštěno % úspěšnosti (H5 podpořena).</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1667,7 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Na obrazovce „Konec“ psovod tlačítkem „Nahrát video“ přiloží video z tréninku, takže už neleží odpojené v galerii.</t>
+          <t>Psovod k tréninku nebo dotazu přiloží odkaz na video. Klienti dnes videa aktivně posílají přes WhatsApp („dělám to dobře?“).</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1598,12 +1682,12 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Stačí v MVP odkaz (YouTube, Disk), nebo nahrání souboru (F-28)? (otázka 6)</t>
+          <t>Stačí odkaz (YouTube, Disk)? Video natočené telefonem pošle klient do WhatsAppu snáz než přes odkaz. (FB2 otázka 9)</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -1611,6 +1695,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1630,7 +1715,7 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Na detailu psa jsou „Aktivity“: odcvičené tréninky po dnech se záznamy, jde porovnat, co fungovalo.</t>
+          <t>Na detailu psa jsou předchozí zadání a odcvičené tréninky. Klient se k nim vrací, trenér spíš ne.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1645,7 +1730,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H30" s="5" t="n"/>
@@ -1654,6 +1739,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1683,7 +1769,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -1693,12 +1779,17 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Jen pokud se bude zadávat % úspěšnosti (otázka 3).</t>
+          <t>Bez % úspěšnosti není co vykreslit (H5).</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Nice to have → Mimo rozsah</t>
         </is>
       </c>
     </row>
@@ -1744,6 +1835,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1787,6 +1879,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1801,12 +1894,12 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Komentáře k tréninku</t>
+          <t>Dotaz k úkolu (vlákno)</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Psovod pošle s tréninkem komentář, trenér mu odpoví ve vlákně a reaguje na video. Nahrazuje WhatsApp.</t>
+          <t>Psovod položí dotaz přímo u úkolu, trenér odpoví. Někdy stačí „děláš to super, pokračuj“, jindy jde o dialog. Trenér hned vidí, ke kterému cviku dotaz patří.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1821,17 +1914,22 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Kde psovod odpověď trenéra uvidí? (otázka 9)</t>
+          <t>Trenérce WhatsApp stačí. Přejdou trenéři na vlákno v aplikaci? Kde psovod odpověď uvidí? (FB2 otázka 7)</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Přeformulováno: z „nahrazuje WhatsApp“ na dotaz u úkolu.</t>
         </is>
       </c>
     </row>
@@ -1877,6 +1975,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1914,12 +2013,17 @@
           <t>Tým</t>
         </is>
       </c>
-      <c r="H36" s="5" t="n"/>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Má smysl, jen když trenér aplikaci otevírá, viz F-33. (FB2 otázka 7)</t>
+        </is>
+      </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -1934,22 +2038,22 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Upozornění</t>
+          <t>Upozornění trenéra e-mailem</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Psovod nebo trenér se dozví o novém komentáři, záznamu nebo změně plánu.</t>
+          <t>Trenér dostane e-mail, když klient položí dotaz nebo pošle záznam. Bez toho dotaz neuvidí a klient se vrátí na WhatsApp. Ostatní upozornění později.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
@@ -1959,12 +2063,17 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>E-mail, nebo stačí upozornění v aplikaci?</t>
+          <t>Stačí e-mail, nebo je potřeba push notifikace (PWA)? (FB2 otázka 7)</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>Nice to have → MVP (zúženo na upozornění trenéra).</t>
         </is>
       </c>
     </row>
@@ -2010,6 +2119,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -2053,6 +2163,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -2100,6 +2211,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -2143,6 +2255,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -2186,6 +2299,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -2229,6 +2343,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -2276,6 +2391,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -2319,6 +2435,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -2362,6 +2479,7 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -2381,7 +2499,7 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Psovod otevře dnešní trénink a prochází cviky jeden po druhém („Aktuální cvik 3/20“), na konci přejde na obrazovku „Konec“.</t>
+          <t>Psovod na place otevře zadání a prochází cviky jeden po druhém („Aktuální cvik 3/20“): princip, dílčí kroky, kritérium a na co si dát pozor. Na konci přejde na zápis tréninku.</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2396,12 +2514,12 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>Znamenají šipky další cvik v dnešním tréninku, nebo posun v plánu (F-14)?</t>
+          <t>Klienti dnes „stojí na place a neví, která bije“. Znamenají šipky další cvik v dnešním tréninku, nebo posun v plánu (F-14)?</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
@@ -2409,50 +2527,215 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>Doplněn obsah cviku: princip, kroky, kritérium.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="n"/>
-      <c r="B48" s="5" t="n"/>
-      <c r="C48" s="5" t="n"/>
-      <c r="D48" s="5" t="n"/>
-      <c r="E48" s="5" t="n"/>
-      <c r="F48" s="5" t="n"/>
-      <c r="G48" s="5" t="n"/>
-      <c r="H48" s="5" t="n"/>
-      <c r="I48" s="5" t="n"/>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>F-44</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Plán tréninku</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Video ukázka u cviku</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Trenér nebo psovod přiloží k cviku odkaz na video z lekce, jak má cvik vypadat. Respondentka se jako klientka k videím vrací často.</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Psovod, trenér</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Nice to have</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>Kdo na lekci natáčí? Stačí odkaz? (FB2 otázka 9)</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>Nové (rozhovor).</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="n"/>
-      <c r="B49" s="5" t="n"/>
-      <c r="C49" s="5" t="n"/>
-      <c r="D49" s="5" t="n"/>
-      <c r="E49" s="5" t="n"/>
-      <c r="F49" s="5" t="n"/>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="5" t="n"/>
-      <c r="I49" s="5" t="n"/>
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>F-45</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Zpětná vazba</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Okolnosti u dotazu</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>U dotazu psovod rovnou vyplní, na co se trenér stejně doptá: jak pes spal, jestli se to stalo poprvé nebo opakovaně, jak se tvářil. Ušetří kolo doptávání.</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Psovod</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Nice to have</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>Které okolnosti trenéři potřebují? Neodradí to klienta od dotazu? (FB2 otázka 8)</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>Nové (rozhovor).</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="n"/>
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="5" t="n"/>
-      <c r="I50" s="5" t="n"/>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>F-46</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Pes a disciplíny</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Vlastní poznámky psovoda</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Psovod si k psovi a disciplíně zapisuje poznámky ze seminářů a plán do budoucna, i od trenérů mimo aplikaci. Dnes papírový deník pro každého psa a sport.</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Psovod</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Nice to have</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>Je psovod bez trenéra cílová skupina? (FB2 otázka 10)</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>Nové (rozhovor).</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n"/>
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="5" t="n"/>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="5" t="n"/>
-      <c r="G51" s="5" t="n"/>
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>F-47</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Plán tréninku</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Aktuální zadání u psa</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Psovod na detailu psa vidí aktuální zadání od trenéra (z poslední lekce) a vrací se k němu, když neví, co cvičit. Funguje i bez kalendáře.</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Psovod</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Rozhovor</t>
+        </is>
+      </c>
       <c r="H51" s="5" t="n"/>
-      <c r="I51" s="5" t="n"/>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>Nové: náhrada za ztracené poznámky z lekce.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
@@ -2464,6 +2747,7 @@
       <c r="G52" s="5" t="n"/>
       <c r="H52" s="5" t="n"/>
       <c r="I52" s="5" t="n"/>
+      <c r="J52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -2475,6 +2759,7 @@
       <c r="G53" s="5" t="n"/>
       <c r="H53" s="5" t="n"/>
       <c r="I53" s="5" t="n"/>
+      <c r="J53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
@@ -2486,6 +2771,7 @@
       <c r="G54" s="5" t="n"/>
       <c r="H54" s="5" t="n"/>
       <c r="I54" s="5" t="n"/>
+      <c r="J54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
@@ -2497,6 +2783,7 @@
       <c r="G55" s="5" t="n"/>
       <c r="H55" s="5" t="n"/>
       <c r="I55" s="5" t="n"/>
+      <c r="J55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n"/>
@@ -2508,6 +2795,7 @@
       <c r="G56" s="5" t="n"/>
       <c r="H56" s="5" t="n"/>
       <c r="I56" s="5" t="n"/>
+      <c r="J56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
@@ -2519,6 +2807,7 @@
       <c r="G57" s="5" t="n"/>
       <c r="H57" s="5" t="n"/>
       <c r="I57" s="5" t="n"/>
+      <c r="J57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n"/>
@@ -2530,6 +2819,7 @@
       <c r="G58" s="5" t="n"/>
       <c r="H58" s="5" t="n"/>
       <c r="I58" s="5" t="n"/>
+      <c r="J58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
@@ -2541,6 +2831,7 @@
       <c r="G59" s="5" t="n"/>
       <c r="H59" s="5" t="n"/>
       <c r="I59" s="5" t="n"/>
+      <c r="J59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
@@ -2552,9 +2843,15 @@
       <c r="G60" s="5" t="n"/>
       <c r="H60" s="5" t="n"/>
       <c r="I60" s="5" t="n"/>
+      <c r="J60" s="5" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I60"/>
+  <autoFilter ref="A4:J60"/>
+  <conditionalFormatting sqref="A5:J60">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$F5="MVP"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="F5:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"MVP,Nice to have,Mimo rozsah"</formula1>
@@ -2715,7 +3012,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Trenér skládá plán z cviků a sekvencí, s návratem, přeskočením a větvením.</t>
+          <t>Trenér zapíše zadání z lekce: cviky, dílčí kroky a kritéria. Při chybě návrat o krok nebo mezikrok.</t>
         </is>
       </c>
       <c r="C8" s="5">
@@ -2740,7 +3037,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Kalendář s tréninky všech psů na celý týden.</t>
+          <t>Psovod si úkoly ze zadání rozvrhne do týdne, tréninky všech psů v jednom kalendáři.</t>
         </is>
       </c>
       <c r="C9" s="5">
@@ -2765,7 +3062,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Psovod projde trénink a odešle video a komentář.</t>
+          <t>Psovod na place projde zadání a zapíše, jak to šlo, případně s videem.</t>
         </is>
       </c>
       <c r="C10" s="5">
@@ -2790,7 +3087,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Trenér vidí, co klienti odcvičili, a reaguje na to.</t>
+          <t>Psovod se zeptá přímo u úkolu, trenér dostane upozornění a odpoví.</t>
         </is>
       </c>
       <c r="C11" s="5">

</xml_diff>

<commit_message>
docs: převzetí návrhů z PR #4
Podle doporučení autora PR #4 (MartinIndra02):
- varianta B Lean Canvasu jako samostatný dokument (lean-canvas-varianta-b.md), sladěná s verzí 1.3
- otázka 0 (kdo aplikaci používá první) v otazky-fb2.md a v plánu
- jeho změny priorit (F-15, % úspěšnosti, F-46, F-18) jen jako alternativní návrhy u otázek na FB 2, breakdown beze změny
- podbarvení MVP řádků v feature-breakdown.xlsx (podmíněné formátování)
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -140,6 +140,16 @@
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2EFDA"/>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -2659,6 +2669,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:I60"/>
+  <conditionalFormatting sqref="A5:I60">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$F5="MVP"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="F5:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"MVP,Nice to have,Mimo rozsah"</formula1>

</xml_diff>

<commit_message>
docs: jeden model po FB2, ceník a šablona user story
PO na FB2 potvrdil, že psovod může aplikaci používat i sám a zve
vždycky trenér. Lean Canvas 1.4 (md i docx) nahrazuje verzi 1.3
i variantu B. Tarify Solo/Pro nahradila platba za aktivního klienta
(3 zdarma, 49 Kč za dalšího, strop 1 490 Kč) včetně přepočtu
v nákladové struktuře. Breakdown (nové F-47 a F-48), sitemapa,
otázky na FB2 a upravený plán sladěné. Šablona issue pro user stories.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature breakdown" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epicy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Návod" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Feature breakdown" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Epicy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Návod" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature breakdown'!$A$4:$I$60</definedName>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -444,7 +444,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tým 5 · aktualizace 9. 10. 2026 po rozhovoru s trenérkou a FB1. „Odsouhlaseno“ = rozhodl upravený plán nebo PO ve FB1, „Navrženo“ = k projednání. „FB2, otázka N“ odkazuje na otazky-fb2.md. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
+          <t>Tým 5 · aktualizace 9. 10. 2026 po rozhovoru s trenérkou, FB1 a FB2 (Lean Canvas 1.4: psovod může aplikaci používat i sám, zve vždycky trenér). „Odsouhlaseno“ = rozhodl upravený plán nebo PO ve FB1 či FB2, „Navrženo“ = k projednání. „FB2, otázka N“ odkazuje na otazky-fb2.md. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
         </is>
       </c>
     </row>
@@ -513,7 +513,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Psovod i trenér si založí účet e-mailem a heslem. Bez účtu se klient s trenérem nepropojí.</t>
+          <t>Psovod i trenér si založí účet e-mailem a heslem. Psovod se může registrovat sám, bez pozvánky, a vést si deník psa. Trenér si při registraci zvolí trenérský účet.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (UP): platí trenér, psovod se registruje přes jeho pozvánku a má aplikaci zdarma.</t>
+          <t>Rozhodnuto (FB2): psovod se registruje i bez pozvánky a má aplikaci zdarma, platí jen trenér.</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Trenér pošle klientovi pozvánku e-mailem nebo mu předá kód (třeba na lekci). Aplikaci platí trenér, proto zve on.</t>
+          <t>Trenér pošle klientovi pozvánku e-mailem nebo mu předá kód (třeba na lekci). Tím mu nabízí placenou podporu mezi lekcemi: zadání v aplikaci a reakce na záznamy.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Klient na úvodní obrazovce zvolí „Mám pozvánku“, zadá kód nebo otevře odkaz, zaregistruje se a propojí se s trenérem.</t>
+          <t>Klient na úvodní obrazovce zvolí „Mám pozvánku“, zadá kód nebo otevře odkaz, zaregistruje se a propojí se s trenérem. Psovod, který už účet má, zadá kód v profilu. Po přijetí vybere psy, které s trenérem sdílí.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Kód platí 7 dní (návrh týmu).</t>
+          <t>Kód platí 7 dní (návrh týmu). Přijetí v existujícím účtu rozhodnuto na FB2.</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -1024,7 +1024,11 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H16" s="5" t="n"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Rozhodnuto (FB2): v MVP zve jen trenér. Psovod může aplikaci používat i sám, trenéra ale nezve.</t>
+        </is>
+      </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1049,12 +1053,12 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Trenér založí pro psa klienta cíl v disciplíně, dlouhodobý (spolehlivá chůze u nohy) i drobný trik (pac). Plán začíná principem: čeho docílit a na co si dát pozor. Trenérka v rozhovoru zadává nejdřív princip, pak cviky.</t>
+          <t>Trenér pro psa klienta nebo psovod pro svého psa založí cíl v disciplíně, dlouhodobý (spolehlivá chůze u nohy) i drobný trik (pac). Plán začíná principem: čeho docílit a na co si dát pozor. Trenérka v rozhovoru zadává nejdřív princip, pak cviky.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1101,7 +1105,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1148,7 +1152,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1191,7 +1195,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1285,7 +1289,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1355,22 +1359,22 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>F-19</t>
+          <t>F-47</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Týdenní rozvrh</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Týdenní kalendář</t>
+          <t>Poznámky z lekce a semináře</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Aktuální týden po dnech, tréninky všech psů najednou, barevně podle psa. Po kliknutí na den karta tréninku se seznamem cviků.</t>
+          <t>Psovod si k psovi zapíše poznámky z lekce nebo semináře (deník psa), aby doma věděl, co trenér říkal, i když zadání nedostal v aplikaci. Respondentka jako klientka: po semináři „co sis zaznamenala, to máš“.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1385,10 +1389,14 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="n"/>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Rozhodnuto (FB2): deník psa je součást produktu. Vidí poznámky trenér? Návrh týmu: ne.</t>
+        </is>
+      </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
@@ -1398,7 +1406,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>F-20</t>
+          <t>F-19</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1408,17 +1416,17 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Naplánování tréninku na den</t>
+          <t>Týdenní kalendář</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Tréninky se zařadí do dnů v týdnu a období (od–do). Rozvrh se zobrazuje v týdnech a dnech jako v aplikaci Runna.</t>
+          <t>Aktuální týden po dnech, tréninky všech psů najednou, barevně podle psa. Po kliknutí na den karta tréninku se seznamem cviků.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Trenér, psovod</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -1431,21 +1439,17 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Kdo zařazuje tréninky do dnů, trenér, nebo psovod? (FB2, otázka 2)</t>
-        </is>
-      </c>
+      <c r="H25" s="5" t="n"/>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>F-21</t>
+          <t>F-20</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1455,17 +1459,17 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Přesunout, nebo přeskočit trénink</t>
+          <t>Naplánování tréninku na den</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Když trénink v daný den neproběhne, psovod ho jedním krokem přesune na jiný den či týden, nebo ho přeskočí, aby nevznikala lavina nedodělků (vzor Runna).</t>
+          <t>Tréninky se zařadí do dnů v týdnu a období (od–do). Rozvrh se zobrazuje v týdnech a dnech jako v aplikaci Runna.</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -1480,19 +1484,19 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Co se stane s přeskočeným cvikem v plánu a vidí to trenér? (FB2, otázka 4)</t>
+          <t>Kdo zařazuje do dnů tréninky z cíle od trenéra, trenér, nebo psovod? (FB2, otázka 2). Svůj vlastní cíl si psovod naplánuje sám.</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>F-22</t>
+          <t>F-21</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1502,12 +1506,12 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Přepínání týdnů</t>
+          <t>Přesunout, nebo přeskočit trénink</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Zpět (co se odcvičilo) i dopředu (plánování).</t>
+          <t>Když trénink v daný den neproběhne, psovod ho jedním krokem přesune na jiný den či týden, nebo ho přeskočí, aby nevznikala lavina nedodělků (vzor Runna).</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1522,20 +1526,24 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Co se stane s přeskočeným cvikem v plánu a vidí to trenér? (FB2, otázka 4)</t>
+        </is>
+      </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>F-23</t>
+          <t>F-22</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1545,12 +1553,12 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Zanedbané disciplíny</t>
+          <t>Přepínání týdnů</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Upozornění, že některá disciplína tento týden nemá trénink. Neodcvičené tréninky řeší F-21.</t>
+          <t>Zpět (co se odcvičilo) i dopředu (plánování).</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1560,19 +1568,15 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>Více disciplín trenérce práci navíc nedělá (H1 oslabena).</t>
-        </is>
-      </c>
+          <t>Předpoklad týmu</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="n"/>
       <c r="I28" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1582,22 +1586,22 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>F-43</t>
+          <t>F-23</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Týdenní rozvrh</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Průchod tréninkem</t>
+          <t>Zanedbané disciplíny</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Psovod otevře dnešní trénink a prochází cviky jeden po druhém („Aktuální cvik 3/20“), na konci přejde na obrazovku „Konec“.</t>
+          <t>Upozornění, že některá disciplína tento týden nemá trénink. Neodcvičené tréninky řeší F-21.</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1607,17 +1611,17 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Šipky = další cvik v dnešním tréninku. Každý cvik ukazuje instrukci a kritérium (F-13).</t>
+          <t>Více disciplín trenérce práci navíc nedělá (H1 oslabena).</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -1629,7 +1633,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>F-24</t>
+          <t>F-43</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1639,12 +1643,12 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Odeslání tréninku</t>
+          <t>Průchod tréninkem</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Na obrazovce „Konec“ psovod zadá % úspěšnosti, rychlé hodnocení (soustředění, opakované chyby) a poznámku a odešle trénink trenérovi. Rychle, z mobilu.</t>
+          <t>Psovod otevře dnešní trénink a prochází cviky jeden po druhém („Aktuální cvik 3/20“), na konci přejde na obrazovku „Konec“.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1659,12 +1663,12 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Za cvik, nebo za celý trénink? Jak má psovod % určit? Trenérka měří úspěch kvalitativně (H5). (FB2, otázka 3)</t>
+          <t>Šipky = další cvik v dnešním tréninku. Každý cvik ukazuje instrukci a kritérium (F-13).</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -1676,7 +1680,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>F-25</t>
+          <t>F-24</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1686,12 +1690,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Video z tréninku</t>
+          <t>Odeslání tréninku</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Na obrazovce „Konec“ psovod vloží odkaz na video z tréninku (YouTube unlisted, cloud), takže video už neleží odpojené v galerii.</t>
+          <t>Na obrazovce „Konec“ psovod zadá % úspěšnosti, rychlé hodnocení (soustředění, opakované chyby) a poznámku a odešle trénink trenérovi. Psovod bez trenéra si záznam uloží do deníku. Rychle, z mobilu.</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1711,19 +1715,19 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Jak klientům vložení odkazu usnadnit? (FB2, otázka 11)</t>
+          <t>Za cvik, nebo za celý trénink? Jak má psovod % určit? Trenérka měří úspěch kvalitativně (H5). (FB2, otázka 3)</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>F-44</t>
+          <t>F-25</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1733,12 +1737,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Kontext k záznamu</t>
+          <t>Video z tréninku</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Psovod u záznamu volitelně vyplní okolnosti (jak pes spal, prostředí, jestli se chyba opakuje), na které se trenérka jinak doptává.</t>
+          <t>Na obrazovce „Konec“ psovod vloží odkaz na video z tréninku (YouTube unlisted, cloud), takže video už neleží odpojené v galerii.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1748,25 +1752,29 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Jak klientům vložení odkazu usnadnit? (FB2, otázka 11)</t>
+        </is>
+      </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>F-26</t>
+          <t>F-44</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1776,27 +1784,27 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Historie tréninků psa</t>
+          <t>Kontext k záznamu</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Na detailu psa jsou „Aktivity“: odcvičené tréninky po dnech s videi a odpověďmi trenéra. Hodnota hlavně pro psovoda, který se k videím a zpětné vazbě vrací (trenérka ne).</t>
+          <t>Psovod u záznamu volitelně vyplní okolnosti (jak pes spal, prostředí, jestli se chyba opakuje), na které se trenérka jinak doptává.</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H33" s="5" t="n"/>
@@ -1809,7 +1817,7 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>F-27</t>
+          <t>F-26</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -1819,12 +1827,12 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Graf vývoje úspěšnosti</t>
+          <t>Historie tréninků psa</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Vývoj % v čase u psa nebo plánu.</t>
+          <t>Na detailu psa jsou „Aktivity“: odcvičené tréninky po dnech s videi a odpověďmi trenéra. Hodnota hlavně pro psovoda, který se k videím a zpětné vazbě vrací (trenérka ne).</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1834,19 +1842,15 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Mimo rozsah</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
-        </is>
-      </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>Úspěch se v praxi číslem neměří (H5 podpořena).</t>
-        </is>
-      </c>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="n"/>
       <c r="I34" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1856,7 +1860,7 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>F-28</t>
+          <t>F-27</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1866,17 +1870,17 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Nahrávání videí na náš server</t>
+          <t>Graf vývoje úspěšnosti</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Vlastní úložiště videí je drahé, v MVP ho nestavíme (viz F-25, otázka 6).</t>
+          <t>Vývoj % v čase u psa nebo plánu.</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -1886,20 +1890,24 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H35" s="5" t="n"/>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Úspěch se v praxi číslem neměří (H5 podpořena).</t>
+        </is>
+      </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>F-29</t>
+          <t>F-28</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -1909,12 +1917,12 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Napojení na Stravu</t>
+          <t>Nahrávání videí na náš server</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Import canicrossových běhů z běžeckých aplikací.</t>
+          <t>Vlastní úložiště videí je drahé, v MVP ho nestavíme (viz F-25, otázka 6).</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1935,39 +1943,39 @@
       <c r="H36" s="5" t="n"/>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>F-30</t>
+          <t>F-29</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Zpětná vazba</t>
+          <t>Záznam tréninku</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Komentáře k tréninku</t>
+          <t>Napojení na Stravu</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Psovod pošle s tréninkem komentář, trenér mu odpoví ve vlákně pod konkrétním tréninkem a reaguje na video. Vlákno unese dialog i doptávání (jak pes spal, jestli se chyba opakuje). Nahrazuje WhatsApp.</t>
+          <t>Import canicrossových běhů z běžeckých aplikací.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
@@ -1978,14 +1986,14 @@
       <c r="H37" s="5" t="n"/>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>F-31</t>
+          <t>F-30</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -1995,17 +2003,17 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Seznam klientů</t>
+          <t>Komentáře k tréninku</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Trenér vidí své klienty (jméno, e-mail) a přes ně jejich psy, plány a odcvičené tréninky.</t>
+          <t>Psovod pošle s tréninkem komentář, trenér mu odpoví ve vlákně pod konkrétním tréninkem a reaguje na video. Vlákno unese dialog i doptávání (jak pes spal, jestli se chyba opakuje). Nahrazuje WhatsApp.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -2018,11 +2026,7 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr">
-        <is>
-          <t>Potvrzeno (PO, FB1): horní přehled svěřenců odpovídá pohledu trenéra.</t>
-        </is>
-      </c>
+      <c r="H38" s="5" t="n"/>
       <c r="I38" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
@@ -2032,7 +2036,7 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>F-32</t>
+          <t>F-31</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -2042,12 +2046,12 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Čeká na reakci</t>
+          <t>Seznam klientů</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Fronta dotazů a záznamů od klientů, na které trenér ještě neodpověděl. Slouží jako pomocník, ne kontrola plnění: trenérka od klientů nic nevyžaduje a pokrok pozná na další lekci.</t>
+          <t>Trenér vidí své klienty (jméno, e-mail) a přes ně jejich psy, plány a odcvičené tréninky.</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2062,20 +2066,24 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Potvrzeno (PO, FB1): horní přehled svěřenců odpovídá pohledu trenéra.</t>
+        </is>
+      </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>F-33</t>
+          <t>F-32</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -2085,17 +2093,17 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Štítek „nová odpověď“</t>
+          <t>Čeká na reakci</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Psovod v Týdnu a u tréninku vidí, že mu trenér odpověděl; trenér vidí nové záznamy. Bez toho psovod odpověď nenajde.</t>
+          <t>Fronta dotazů a záznamů od klientů, na které trenér ještě neodpověděl. Slouží jako pomocník, ne kontrola plnění: trenérka od klientů nic nevyžaduje a pokrok pozná na další lekci.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
@@ -2118,7 +2126,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>F-46</t>
+          <t>F-33</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -2128,12 +2136,12 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>E-mailová upozornění</t>
+          <t>Štítek „nová odpověď“</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Psovod nebo trenér dostane e-mail o nové odpovědi, záznamu nebo změně plánu.</t>
+          <t>Psovod v Týdnu a u tréninku vidí, že mu trenér odpověděl; trenér vidí nové záznamy. Bez toho psovod odpověď nenajde.</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2143,19 +2151,15 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>Stačí upozornění v aplikaci, nebo je potřeba i e-mail? (FB2, otázka 5)</t>
-        </is>
-      </c>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="n"/>
       <c r="I41" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -2165,22 +2169,22 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>F-34</t>
+          <t>F-46</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Tržiště a platby</t>
+          <t>Zpětná vazba</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Prodej a nákup plánů, hodnocení</t>
+          <t>E-mailová upozornění</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Veřejné tržiště plánů z původního briefu.</t>
+          <t>Psovod nebo trenér dostane e-mail o nové odpovědi, záznamu nebo změně plánu.</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2190,25 +2194,29 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Mimo rozsah</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H42" s="5" t="n"/>
+          <t>Předpoklad týmu</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Stačí upozornění v aplikaci, nebo je potřeba i e-mail? (FB2, otázka 5)</t>
+        </is>
+      </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>F-35</t>
+          <t>F-34</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -2218,17 +2226,17 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Předplatné a platby</t>
+          <t>Prodej a nákup plánů, hodnocení</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Budoucí předplatné pro trenéry, tento semestr bez plateb.</t>
+          <t>Veřejné tržiště plánů z původního briefu.</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -2251,54 +2259,54 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>F-36</t>
+          <t>F-35</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Technický základ</t>
+          <t>Tržiště a platby</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Staging a CI/CD</t>
+          <t>Předplatné a platby</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Každá změna se otestuje a nasadí na staging, kde ji PO uvidí dřív než uživatelé.</t>
+          <t>Trenér platí za aktivního klienta: 3 zdarma, pak 49 Kč měsíčně za každého dalšího, strop 1 490 Kč měsíčně. Psovod 0 Kč. Tento semestr platby nestavíme.</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>Kdo bude mít přístup na staging?</t>
+          <t>Ceník je návrh týmu, viz lean-canvas.md a nakladova-struktura.xlsx (FB2, otázka 8).</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>F-37</t>
+          <t>F-36</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -2308,12 +2316,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Automatické testy</t>
+          <t>Staging a CI/CD</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Hlavní obrana proti chybám od agenta, hlavně v logice nelineárního plánu.</t>
+          <t>Každá změna se otestuje a nasadí na staging, kde ji PO uvidí dřív než uživatelé.</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2331,7 +2339,11 @@
           <t>Tým</t>
         </is>
       </c>
-      <c r="H45" s="5" t="n"/>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>Kdo bude mít přístup na staging?</t>
+        </is>
+      </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -2341,7 +2353,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>F-38</t>
+          <t>F-37</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -2351,12 +2363,12 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Oprávnění</t>
+          <t>Automatické testy</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Kdo vidí a upravuje psa, plán, záznamy a komentáře (psovod, trenér, cizí).</t>
+          <t>Hlavní obrana proti chybám od agenta, hlavně v logice nelineárního plánu.</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2384,7 +2396,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>F-39</t>
+          <t>F-38</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -2394,17 +2406,17 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Osobní údaje a smazání účtu</t>
+          <t>Oprávnění</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Souhlas se zpracováním, smazání účtu včetně dat.</t>
+          <t>Kdo vidí a upravuje psa, plán, záznamy a komentáře (psovod, trenér, cizí).</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -2427,7 +2439,7 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>F-40</t>
+          <t>F-39</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
@@ -2437,12 +2449,12 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Použitelnost na mobilu</t>
+          <t>Osobní údaje a smazání účtu</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Psovod zapisuje venku po tréninku, aplikace musí fungovat na telefonu.</t>
+          <t>Souhlas se zpracováním, smazání účtu včetně dat.</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2457,24 +2469,20 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>Rozhodnuto: responzivní webová aplikace (optimalizovaná pro mobil / PWA). Nativní aplikace v App Store / Google Play mimo rozsah pilotu.</t>
-        </is>
-      </c>
+          <t>Tým</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="n"/>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>F-41</t>
+          <t>F-40</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -2484,17 +2492,17 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Zálohy dat</t>
+          <t>Použitelnost na mobilu</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Pravidelná záloha databáze, aby historie tréninků nezmizela.</t>
+          <t>Psovod zapisuje venku po tréninku, aplikace musí fungovat na telefonu.</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -2504,20 +2512,24 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>Rozhodnuto: responzivní webová aplikace (optimalizovaná pro mobil / PWA). Nativní aplikace v App Store / Google Play mimo rozsah pilotu.</t>
+        </is>
+      </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>F-42</t>
+          <t>F-41</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
@@ -2527,12 +2539,12 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Monitoring a logy</t>
+          <t>Zálohy dat</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>O chybě se dozvíme dřív než uživatel.</t>
+          <t>Pravidelná záloha databáze, aby historie tréninků nezmizela.</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2542,7 +2554,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -2558,26 +2570,94 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n"/>
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="5" t="n"/>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="5" t="n"/>
-      <c r="G51" s="5" t="n"/>
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>F-42</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Technický základ</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Monitoring a logy</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>O chybě se dozvíme dřív než uživatel.</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Tým</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Nice to have</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Tým</t>
+        </is>
+      </c>
       <c r="H51" s="5" t="n"/>
-      <c r="I51" s="5" t="n"/>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>Navrženo</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="n"/>
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="5" t="n"/>
-      <c r="D52" s="5" t="n"/>
-      <c r="E52" s="5" t="n"/>
-      <c r="F52" s="5" t="n"/>
-      <c r="G52" s="5" t="n"/>
-      <c r="H52" s="5" t="n"/>
-      <c r="I52" s="5" t="n"/>
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>F-48</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Technický základ</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Odesílání e-mailů</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Aplikace posílá e-maily: pozvánku klienta (F-08) a obnovu hesla (F-02). Klient je nevidí, ale bez nich tyto features nefungují.</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Tým</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Tým</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Jakou službu použít a kdo ji zaplatí?</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Navrženo</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -2666,6 +2746,28 @@
       <c r="G60" s="5" t="n"/>
       <c r="H60" s="5" t="n"/>
       <c r="I60" s="5" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n"/>
+      <c r="B61" s="5" t="n"/>
+      <c r="C61" s="5" t="n"/>
+      <c r="D61" s="5" t="n"/>
+      <c r="E61" s="5" t="n"/>
+      <c r="F61" s="5" t="n"/>
+      <c r="G61" s="5" t="n"/>
+      <c r="H61" s="5" t="n"/>
+      <c r="I61" s="5" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="n"/>
+      <c r="B62" s="5" t="n"/>
+      <c r="C62" s="5" t="n"/>
+      <c r="D62" s="5" t="n"/>
+      <c r="E62" s="5" t="n"/>
+      <c r="F62" s="5" t="n"/>
+      <c r="G62" s="5" t="n"/>
+      <c r="H62" s="5" t="n"/>
+      <c r="I62" s="5" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:I60"/>
@@ -2809,7 +2911,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Trenér pozve klienta a propojí se s jeho psem.</t>
+          <t>Trenér pozve psovoda a propojí se s jeho psem.</t>
         </is>
       </c>
       <c r="C7" s="5">
@@ -2834,7 +2936,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Trenér skládá plán z cviků a sekvencí, s návratem, přeskočením a větvením.</t>
+          <t>Psovod nebo trenér skládá plán z cviků a sekvencí, s návratem, přeskočením a větvením.</t>
         </is>
       </c>
       <c r="C8" s="5">

</xml_diff>

<commit_message>
docs: úklid výstupů Sprintu 1 po FB2
- rozcestník docs/vystupy/README.md: sedm výstupů Sprintu 1 a kde jsou
- po-feedback.md: FB1 beze změny a nově rozhodnutí z FB2 (podle PR #5)
- otazky-na-po.md (dřív otazky-fb2.md): jen otevřené otázky, nová otázka 12 k F-47
- rozhovor/vysledky.md: tabulka zjištění Z1–Z11 s dopadem na produkt (přesunuto z plánu úprav)
- sitemapa: nový wireframe Vytvořit psa, seznam úprav wireframů (přesunuto z plánu úprav), opravené odkazy, SVG bez varianty B
- breakdown: F-11 mimo rozsah (FB2: psovod trenéra nezve), F-47 do epicu Pes a disciplíny, barva psa u F-04, účely epiců, poznámka k F-48
- nákladová struktura: poznámka k nákladům na e-maily
- smazáno: _archiv, plan-uprav-po-fb1.md, otazky-na-klienta.md, rozhovor/poznamky.md (obsah je v historii a v ostatních dokumentech)
- původní brief přesunut do docs/materialy
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Feature breakdown" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Epicy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Návod" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature breakdown" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epicy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Návod" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature breakdown'!$A$4:$I$60</definedName>
@@ -444,7 +444,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tým 5 · aktualizace 9. 10. 2026 po rozhovoru s trenérkou, FB1 a FB2 (Lean Canvas 1.4: psovod může aplikaci používat i sám, zve vždycky trenér). „Odsouhlaseno“ = rozhodl upravený plán nebo PO ve FB1 či FB2, „Navrženo“ = k projednání. „FB2, otázka N“ odkazuje na otazky-fb2.md. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
+          <t>Tým 5 · aktualizace 9. 10. 2026 po rozhovoru s trenérkou, FB1 a FB2 (Lean Canvas 1.4: psovod může aplikaci používat i sám, zve vždycky trenér). „Odsouhlaseno“ = rozhodl upravený plán nebo PO ve FB1 či FB2, „Navrženo“ = k projednání. „FB2, otázka N“ odkazuje na otazky-na-po.md. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Psovod založí psa (jméno, plemeno, fotka). Pes je středem plánu, kalendáře i spolupráce s trenérem.</t>
+          <t>Psovod založí psa (jméno, plemeno, fotka) a vybere mu barvu, podle které ho pozná v kalendáři. Pes je středem plánu, kalendáře i spolupráce s trenérem.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -854,27 +854,27 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>F-08</t>
+          <t>F-47</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Sdílení s trenérem</t>
+          <t>Pes a disciplíny</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Trenér pozve klienta</t>
+          <t>Poznámky z lekce a semináře</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Trenér pošle klientovi pozvánku e-mailem nebo mu předá kód (třeba na lekci). Tím mu nabízí placenou podporu mezi lekcemi: zadání v aplikaci a reakce na záznamy.</t>
+          <t>Psovod si k psovi zapíše poznámky z lekce nebo semináře (deník psa), aby doma věděl, co trenér říkal, i když zadání nedostal v aplikaci. Respondentka jako klientka: po semináři „co sis zaznamenala, to máš“.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (UP): zve trenér e-mailem nebo kódem. Trenér zve člověka, klient po přijetí vybere nebo založí psa.</t>
+          <t>Vidí poznámky trenér? Návrh týmu: ne. (FB2, otázka 12)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>F-09</t>
+          <t>F-08</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -911,17 +911,17 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Přijetí pozvánky („Mám pozvánku“)</t>
+          <t>Trenér pozve klienta</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Klient na úvodní obrazovce zvolí „Mám pozvánku“, zadá kód nebo otevře odkaz, zaregistruje se a propojí se s trenérem. Psovod, který už účet má, zadá kód v profilu. Po přijetí vybere psy, které s trenérem sdílí.</t>
+          <t>Trenér pošle klientovi pozvánku e-mailem nebo mu předá kód (třeba na lekci). Tím mu nabízí placenou podporu mezi lekcemi: zadání v aplikaci a reakce na záznamy.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Kód platí 7 dní (návrh týmu). Přijetí v existujícím účtu rozhodnuto na FB2.</t>
+          <t>Rozhodnuto (UP): zve trenér e-mailem nebo kódem. Trenér zve člověka, klient po přijetí vybere nebo založí psa.</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -948,7 +948,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>F-10</t>
+          <t>F-09</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Odebrání přístupu</t>
+          <t>Přijetí pozvánky („Mám pozvánku“)</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Trenér nebo psovod ukončí spolupráci, trenér psa přestane vidět.</t>
+          <t>Klient na úvodní obrazovce zvolí „Mám pozvánku“, zadá kód nebo otevře odkaz, zaregistruje se a propojí se s trenérem. Psovod, který už účet má, zadá kód v profilu. Po přijetí vybere psy, které s trenérem sdílí.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -978,20 +978,24 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Kód platí 7 dní (návrh týmu). Přijetí v existujícím účtu rozhodnuto na FB2.</t>
+        </is>
+      </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>F-11</t>
+          <t>F-10</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1001,22 +1005,22 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Psovod pozve trenéra</t>
+          <t>Odebrání přístupu</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Obrácený směr: psovod, který už trenéra má, ho pozve do aplikace.</t>
+          <t>Trenér nebo psovod ukončí spolupráci, trenér psa přestane vidět.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1024,11 +1028,7 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Rozhodnuto (FB2): v MVP zve jen trenér. Psovod může aplikaci používat i sám, trenéra ale nezve.</t>
-        </is>
-      </c>
+      <c r="H16" s="5" t="n"/>
       <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1038,32 +1038,32 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>F-12</t>
+          <t>F-11</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku</t>
+          <t>Sdílení s trenérem</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Cíl a plán tréninku</t>
+          <t>Psovod pozve trenéra</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Trenér pro psa klienta nebo psovod pro svého psa založí cíl v disciplíně, dlouhodobý (spolehlivá chůze u nohy) i drobný trik (pac). Plán začíná principem: čeho docílit a na co si dát pozor. Trenérka v rozhovoru zadává nejdřív princip, pak cviky.</t>
+          <t>Obrácený směr: psovod, který už trenéra má, ho pozve do aplikace.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Trenér, psovod</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (PO, FB1): plán musí unést dlouhodobé cíle i drobné triky.</t>
+          <t>Rozhodnuto (FB2): zve vždycky trenér, psovod trenéra nezve. Psovod může aplikaci používat i sám.</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -1085,7 +1085,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>F-13</t>
+          <t>F-12</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1095,12 +1095,12 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Cviky a sekvence cviků</t>
+          <t>Cíl a plán tréninku</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Plán se skládá z bloků „Jednotlivý cvik“ a „Sekvence cviků“. Každý cvik má instrukci a kritérium zvládnutí („sedí, i když kolem letí míčky“), aby klient doma věděl, co přesně cvičit. Blok jde přidat, upravit, smazat nebo vložit jako mezikrok.</t>
+          <t>Trenér pro psa klienta nebo psovod pro svého psa založí cíl v disciplíně, dlouhodobý (spolehlivá chůze u nohy) i drobný trik (pac). Plán začíná principem: čeho docílit a na co si dát pozor. Trenérka v rozhovoru zadává nejdřív princip, pak cviky.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1115,24 +1115,24 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Instrukce a kritérium u cviku jsou z rozhovoru (klienti si ústní zadání nezapamatují). Potvrdit na FB2.</t>
+          <t>Rozhodnuto (PO, FB1): plán musí unést dlouhodobé cíle i drobné triky.</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>F-14</t>
+          <t>F-13</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1142,12 +1142,12 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Posun, návrat a přeskočení</t>
+          <t>Cviky a sekvence cviků</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Je vidět, na kterém cviku pes je. Když nejde („tunel“, opakuje stejnou chybu), vrátí se o krok; když to umí, cvik se přeskočí. O posunu rozhoduje člověk podle chování psa.</t>
+          <t>Plán se skládá z bloků „Jednotlivý cvik“ a „Sekvence cviků“. Každý cvik má instrukci a kritérium zvládnutí („sedí, i když kolem letí míčky“), aby klient doma věděl, co přesně cvičit. Blok jde přidat, upravit, smazat nebo vložit jako mezikrok.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1162,20 +1162,24 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="n"/>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Instrukce a kritérium u cviku jsou z rozhovoru (klienti si ústní zadání nezapamatují). Potvrdit na FB2.</t>
+        </is>
+      </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>F-15</t>
+          <t>F-14</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1185,12 +1189,12 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Rozvětvení cesty</t>
+          <t>Posun, návrat a přeskočení</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Cesta se rozvětví. Pro MVP v jednoduché podobě: krok, který pes nechápe, se rozdělí na dílčí kroky a po jejich zvládnutí se cesta vrací do hlavní linie („nejdřív kousky, pak celek“). Datový model nepřekombinovat (PO, FB1).</t>
+          <t>Je vidět, na kterém cviku pes je. Když nejde („tunel“, opakuje stejnou chybu), vrátí se o krok; když to umí, cvik se přeskočí. O posunu rozhoduje člověk podle chování psa.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1208,11 +1212,7 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>Podobu ukázat na FB2 (otázka 1).</t>
-        </is>
-      </c>
+      <c r="H20" s="5" t="n"/>
       <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
@@ -1222,7 +1222,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>F-16</t>
+          <t>F-15</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1232,17 +1232,17 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Úpravy plánu podle výsledků</t>
+          <t>Rozvětvení cesty</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Psovod i trenér mohou upravit plán v Tvorbě tréninku. Trenér navíc po reakci na odeslaný trénink plán upraví.</t>
+          <t>Cesta se rozvětví. Pro MVP v jednoduché podobě: krok, který pes nechápe, se rozdělí na dílčí kroky a po jejich zvládnutí se cesta vrací do hlavní linie („nejdřív kousky, pak celek“). Datový model nepřekombinovat (PO, FB1).</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (UP): plán upravují psovod i trenér.</t>
+          <t>Podobu ukázat na FB2 (otázka 1).</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -1269,7 +1269,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>F-17</t>
+          <t>F-16</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1279,17 +1279,17 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Dokončení a archiv plánu</t>
+          <t>Úpravy plánu podle výsledků</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Dokončený nebo opuštěný plán zmizí z aktivních, ale zůstane v historii.</t>
+          <t>Psovod i trenér mohou upravit plán v Tvorbě tréninku. Trenér navíc po reakci na odeslaný trénink plán upraví.</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Trenér, psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1299,20 +1299,24 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Rozhodnuto (UP): plán upravují psovod i trenér.</t>
+        </is>
+      </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>F-18</t>
+          <t>F-17</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1322,22 +1326,22 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Kopie plánu / šablona trenéra</t>
+          <t>Dokončení a archiv plánu</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Trenér zkopíruje osvědčený plán k dalšímu psovi.</t>
+          <t>Dokončený nebo opuštěný plán zmizí z aktivních, ale zůstane v historii.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -1345,11 +1349,7 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Dávají trenéři podobné plány více klientům? (FB2, otázka 7)</t>
-        </is>
-      </c>
+      <c r="H23" s="5" t="n"/>
       <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1359,7 +1359,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>F-47</t>
+          <t>F-18</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1369,37 +1369,37 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Poznámky z lekce a semináře</t>
+          <t>Kopie plánu / šablona trenéra</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Psovod si k psovi zapíše poznámky z lekce nebo semináře (deník psa), aby doma věděl, co trenér říkal, i když zadání nedostal v aplikaci. Respondentka jako klientka: po semináři „co sis zaznamenala, to máš“.</t>
+          <t>Trenér zkopíruje osvědčený plán k dalšímu psovi.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
+          <t>Předpoklad týmu</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (FB2): deník psa je součást produktu. Vidí poznámky trenér? Návrh týmu: ne.</t>
+          <t>Dávají trenéři podobné plány více klientům? (FB2, otázka 7)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
         </is>
       </c>
     </row>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>Jakou službu použít a kdo ji zaplatí?</t>
+          <t>Jakou službu použít? Počítáme s bezplatným tarifem e-mailové služby, v cashflow proto bez nákladu.</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Psovod založí psa a oblasti, ve kterých trénuje.</t>
+          <t>Psovod založí psa a oblasti, ve kterých trénuje, a vede si deník psa.</t>
         </is>
       </c>
       <c r="C6" s="5">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Psovod projde trénink a odešle video a komentář.</t>
+          <t>Psovod projde trénink a zapíše, jak šel: hodnocení, poznámku a odkaz na video.</t>
         </is>
       </c>
       <c r="C10" s="5">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Trenér vidí, co klienti odcvičili, a reaguje na to.</t>
+          <t>Trenér odpovídá na dotazy a záznamy klientů ve vlákně u tréninku.</t>
         </is>
       </c>
       <c r="C11" s="5">

</xml_diff>

<commit_message>
docs: zapracování hodnocení Sprintu 1 (Lean Canvas 1.5, breakdown 32 features, komunikace s PO)
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -432,6 +432,8 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.7" customHeight="1">
@@ -444,7 +446,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tým 5 · aktualizace 9. 10. 2026 po rozhovoru s trenérkou, FB1 a FB2 (Lean Canvas 1.4: psovod může aplikaci používat i sám, zve vždycky trenér). „Odsouhlaseno“ = rozhodl upravený plán nebo PO ve FB1 či FB2, „Navrženo“ = k projednání. „FB2, otázka N“ odkazuje na otazky-na-po.md. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
+          <t>Tým 5 · aktualizace 16. 10. 2026 podle hodnocení Sprintu 1: sjednocená granularita. Feature = jedna schopnost produktu, kterou uživatel pozná. Drobné části jsou user stories v GitHubu (sloupec User stories). Sloupec „Dříve“ převádí ID do 9. 10. „Odsouhlaseno“ = rozhodl upravený plán nebo PO (FB1, FB2, zadání sprintu 2 a standup 15. 10.), „Navrženo“ = k projednání. „Otázka N“ odkazuje na otazky-na-po.md.</t>
         </is>
       </c>
     </row>
@@ -494,6 +496,16 @@
           <t>Stav</t>
         </is>
       </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>User stories</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Dříve (ID do 9. 10.)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -508,12 +520,12 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Registrace a přihlášení</t>
+          <t>Registrace, přihlášení a obnova hesla</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Psovod i trenér si založí účet e-mailem a heslem. Psovod se může registrovat sám, bez pozvánky, a vést si deník psa. Trenér si při registraci zvolí trenérský účet.</t>
+          <t>Psovod i trenér si založí účet e-mailem a heslem (trenér volbou „Jsem trenér“), přihlásí se a zapomenuté heslo obnoví přes e-mail. Psovod se může registrovat i bez pozvánky a vést si deník psa sám.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -533,12 +545,22 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (FB2): psovod se registruje i bez pozvánky a má aplikaci zdarma, platí jen trenér.</t>
+          <t>Rozhodnuto (FB2): psovod se registruje i bez pozvánky.</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>#49, #50, #51, #52</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>F-01, F-02</t>
         </is>
       </c>
     </row>
@@ -555,17 +577,17 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Obnova hesla</t>
+          <t>Úvodní stránka</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Zapomenuté heslo si uživatel obnoví přes e-mail.</t>
+          <t>Veřejná stránka, kde návštěvník pochopí, co aplikace dá trenérovi a psovodovi, a proklikne se na registraci, přihlášení nebo pozvánku od trenéra.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Návštěvník</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -575,13 +597,23 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H6" s="5" t="n"/>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>#102</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>nová (PO 14. 10.)</t>
         </is>
       </c>
     </row>
@@ -627,6 +659,16 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>#92</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>F-03</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -641,12 +683,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Profil psa</t>
+          <t>Pes a jeho disciplíny</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Psovod založí psa (jméno, plemeno, fotka) a vybere mu barvu, podle které ho pozná v kalendáři. Pes je středem plánu, kalendáře i spolupráce s trenérem.</t>
+          <t>Psovod založí jednoho i více psů (jméno, plemeno, fotka, barva v kalendáři), přiřadí jim disciplíny z nabídky nebo vlastní, údaje upraví a disciplínu, kterou pes už netrénuje, ukončí. Pes je středem aplikace.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -664,10 +706,24 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n"/>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Rozhodnuto (UP): více psů na účtu psovoda.</t>
+        </is>
+      </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>#53, #54, #55, #56, #57</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>F-04, F-05, F-06, F-07</t>
         </is>
       </c>
     </row>
@@ -684,12 +740,12 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Disciplíny psa</t>
+          <t>Deník psa: poznámky z lekce a semináře</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Psovod psovi přiřadí oblasti — z nabídky (canicross, nosework, poslušnost) nebo vlastní.</t>
+          <t>Psovod si k psovi zapíše poznámky z lekce nebo semináře (deník psa), aby doma věděl, co trenér říkal, i když zadání nedostal v aplikaci. Respondentka jako klientka: po semináři „co sis zaznamenala, to máš“.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -704,13 +760,27 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="n"/>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Vidí poznámky trenér? Návrh týmu: ne (otázka 12).</t>
+        </is>
+      </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>#70</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>F-47</t>
         </is>
       </c>
     </row>
@@ -727,37 +797,47 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Více psů na účtu</t>
+          <t>Vlastní psi trenéra</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Psovod s více psy vidí jejich tréninky v jednom týdnu.</t>
+          <t>Trenér vede v aplikaci i své psy místo papírového deníku (respondentka má 3 psy a deník na každého psa a sport).</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (UP): více psů na účtu psovoda, i pod trenérem zdarma.</t>
+          <t>Chce to trenér? (otázka 6)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>#93</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>F-45</t>
         </is>
       </c>
     </row>
@@ -769,22 +849,22 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Pes a disciplíny</t>
+          <t>Sdílení s trenérem</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Úprava a archivace psa či disciplíny</t>
+          <t>Propojení trenéra s klientem</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Změna údajů, ukončení disciplíny, kterou pes už netrénuje. Historie zůstane.</t>
+          <t>Trenér klientovi vygeneruje kód (třeba na lekci) nebo pošle pozvánku e-mailem. Klient kód zadá, vybere psy, které s trenérem sdílí, a propojí se. Spolupráci jde ukončit, trenér pak psa přestane vidět.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -794,87 +874,107 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="n"/>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Kód platí 7 dní (návrh týmu).</t>
+        </is>
+      </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>#58, #59, #60, #61</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>F-08, F-09, F-10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>F-45</t>
+          <t>F-08</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Pes a disciplíny</t>
+          <t>Sdílení s trenérem</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Vlastní psi trenéra</t>
+          <t>Psovod pozve trenéra</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Trenér vede v aplikaci i své psy místo papírového deníku (respondentka má 3 psy a deník na každého psa a sport).</t>
+          <t>Obrácený směr: psovod, který už trenéra má, ho pozve do aplikace.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Chce to trenér? (FB2, otázka 6)</t>
+          <t>Rozhodnuto (FB2): zve vždycky trenér.</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>F-11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>F-47</t>
+          <t>F-09</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Pes a disciplíny</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Poznámky z lekce a semináře</t>
+          <t>Cíl s cviky a sekvencemi</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Psovod si k psovi zapíše poznámky z lekce nebo semináře (deník psa), aby doma věděl, co trenér říkal, i když zadání nedostal v aplikaci. Respondentka jako klientka: po semináři „co sis zaznamenala, to máš“.</t>
+          <t>Trenér pro psa klienta nebo psovod pro svého psa založí cíl v disciplíně s principem (čeho docílit a na co si dát pozor). Pod cíl skládá cviky s instrukcí a kritériem zvládnutí a sekvence cviků, upravuje je, maže a mění jejich pořadí. Dlouhodobý cíl i drobný trik se zakládají stejně.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -884,44 +984,54 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Vidí poznámky trenér? Návrh týmu: ne. (FB2, otázka 12)</t>
+          <t>Rozhodnuto (PO, FB1): plán unese dlouhodobé cíle i drobné triky.</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>#62, #63, #64, #65</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>F-12, F-13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>F-08</t>
+          <t>F-10</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Sdílení s trenérem</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Trenér pozve klienta</t>
+          <t>Postup plánem</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Trenér pošle klientovi pozvánku e-mailem nebo mu předá kód (třeba na lekci). Tím mu nabízí placenou podporu mezi lekcemi: zadání v aplikaci a reakce na záznamy.</t>
+          <t>Je vidět, na kterém cviku pes je. Když nejde („tunel“, opakuje stejnou chybu), vrátí se o krok nebo se krok rozdělí na dílčí kroky. Když to umí, cvik přeskočí.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -936,39 +1046,49 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (UP): zve trenér e-mailem nebo kódem. Trenér zve člověka, klient po přijetí vybere nebo založí psa.</t>
+          <t>Podoba větvení (otázka 1).</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>#66, #67</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>F-14, F-15</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>F-09</t>
+          <t>F-11</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Sdílení s trenérem</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Přijetí pozvánky („Mám pozvánku“)</t>
+          <t>Úpravy a archiv plánu</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Klient na úvodní obrazovce zvolí „Mám pozvánku“, zadá kód nebo otevře odkaz, zaregistruje se a propojí se s trenérem. Psovod, který už účet má, zadá kód v Účtu. Po přijetí vybere psy, které s trenérem sdílí.</t>
+          <t>Psovod i trenér plán upraví, trenér hlavně po reakci na odeslaný záznam. Dokončený nebo opuštěný cíl zmizí z aktivních, ale zůstane v historii.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér, psovod</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -983,44 +1103,54 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Kód platí 7 dní (návrh týmu). Přijetí v existujícím účtu rozhodnuto na FB2.</t>
+          <t>Rozhodnuto (UP): plán upravují psovod i trenér.</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>#68, #69</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>F-16, F-17</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>F-10</t>
+          <t>F-12</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Sdílení s trenérem</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Odebrání přístupu</t>
+          <t>Kopie plánu / šablona trenéra</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Trenér nebo psovod ukončí spolupráci, trenér psa přestane vidět.</t>
+          <t>Trenér zkopíruje osvědčený plán k dalšímu psovi.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1028,42 +1158,56 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H16" s="5" t="n"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Dávají trenéři podobné plány více klientům? (otázka 7)</t>
+        </is>
+      </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>#94</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>F-18</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>F-11</t>
+          <t>F-13</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Sdílení s trenérem</t>
+          <t>Týdenní rozvrh</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Psovod pozve trenéra</t>
+          <t>Týden s tréninky</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Obrácený směr: psovod, který už trenéra má, ho pozve do aplikace.</t>
+          <t>Psovod vidí tréninky všech psů po dnech, barevně podle psa, a přepíná týdny. Trenér trénink přiřadí ke konkrétnímu dni. Rozvrh po týdnech a dnech jako v aplikaci Runna.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Mimo rozsah</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1073,39 +1217,49 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (FB2): zve vždycky trenér, psovod trenéra nezve. Psovod může aplikaci používat i sám.</t>
+          <t>Rozhodnuto (standup 15. 10.): konkrétní den, ne frekvence.</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>#71, #72, #73</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>F-19, F-20, F-22</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>F-12</t>
+          <t>F-14</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku</t>
+          <t>Týdenní rozvrh</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Cíl a plán tréninku</t>
+          <t>Přesunout, nebo přeskočit trénink</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Trenér pro psa klienta nebo psovod pro svého psa založí cíl v disciplíně, dlouhodobý (spolehlivá chůze u nohy) i drobný trik (pac). Plán začíná principem: čeho docílit a na co si dát pozor. Trenérka v rozhovoru zadává nejdřív princip, pak cviky.</t>
+          <t>Když trénink v daný den neproběhne, psovod ho jedním krokem přesune na jiný den či týden, nebo ho přeskočí, aby nevznikala lavina nedodělků (vzor Runna).</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Trenér, psovod</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1120,129 +1274,163 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto (PO, FB1): plán musí unést dlouhodobé cíle i drobné triky.</t>
+          <t>Co se stane s přeskočeným tréninkem? (otázka 4)</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>#74, #75</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>F-21</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>F-13</t>
+          <t>F-15</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku</t>
+          <t>Týdenní rozvrh</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Cviky a sekvence cviků</t>
+          <t>Duplikace tréninku</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Plán se skládá z bloků „Jednotlivý cvik“ a „Sekvence cviků“. Každý cvik má instrukci a kritérium zvládnutí („sedí, i když kolem letí míčky“), aby klient doma věděl, co přesně cvičit. Blok jde přidat, upravit, smazat nebo vložit jako mezikrok.</t>
+          <t>Trenér zkopíruje naplánovaný trénink na další den, když ho má klient dělat víckrát v týdnu.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Trenér, psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Instrukce a kritérium u cviku jsou z rozhovoru (klienti si ústní zadání nezapamatují). Potvrdit na FB2.</t>
+          <t>PO: do budoucna, teď ne (standup 15. 10.).</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>#103</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>nová (standup 15. 10.)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>F-14</t>
+          <t>F-16</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku</t>
+          <t>Týdenní rozvrh</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Posun, návrat a přeskočení</t>
+          <t>Zanedbané disciplíny</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Je vidět, na kterém cviku pes je. Když nejde („tunel“, opakuje stejnou chybu), vrátí se o krok; když to umí, cvik se přeskočí. O posunu rozhoduje člověk podle chování psa.</t>
+          <t>Upozornění, že některá disciplína tento týden nemá trénink. Neodcvičené tréninky řeší F-21.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Trenér, psovod</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="n"/>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Více disciplín trenérce práci navíc nedělá (H1 oslabena).</t>
+        </is>
+      </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>#95</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>F-23</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>F-15</t>
+          <t>F-17</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku</t>
+          <t>Záznam tréninku</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Rozvětvení cesty</t>
+          <t>Trénink a záznam</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Cesta se rozvětví. Pro MVP v jednoduché podobě: krok, který pes nechápe, se rozdělí na dílčí kroky a po jejich zvládnutí se cesta vrací do hlavní linie („nejdřív kousky, pak celek“). Datový model nepřekombinovat (PO, FB1).</t>
+          <t>Psovod otevře dnešní trénink, prochází cviky s instrukcí a kritériem (šipkami) a na konci zapíše hodnocení, poznámku a odkaz na video. Trenér záznam vidí u psa.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Trenér, psovod</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1257,34 +1445,44 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Podobu ukázat na FB2 (otázka 1).</t>
+          <t>Podoba hodnocení (otázka 3), usnadnění odkazu na video (otázka 11).</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>#76, #77, #78</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>F-43, F-24, F-25</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>F-16</t>
+          <t>F-18</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku</t>
+          <t>Záznam tréninku</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Úpravy plánu podle výsledků</t>
+          <t>Aktivity psa</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Psovod i trenér mohou upravit plán v Tvorbě tréninku. Trenér navíc po reakci na odeslaný trénink plán upraví.</t>
+          <t>Na detailu psa jsou „Aktivity“: odcvičené tréninky po dnech s videi a odpověďmi trenéra. Hodnota hlavně pro psovoda, který se k videím a zpětné vazbě vrací (trenérka ne).</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1302,51 +1500,57 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>Rozhodnuto (UP): plán upravují psovod i trenér.</t>
-        </is>
-      </c>
+      <c r="H22" s="5" t="n"/>
       <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>#79</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>F-26</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>F-17</t>
+          <t>F-19</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku</t>
+          <t>Záznam tréninku</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Dokončení a archiv plánu</t>
+          <t>Kontext k záznamu</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Dokončený nebo opuštěný plán zmizí z aktivních, ale zůstane v historii.</t>
+          <t>Psovod u záznamu volitelně vyplní okolnosti (jak pes spal, prostředí, jestli se chyba opakuje), na které se trenérka jinak doptává.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Trenér, psovod</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
+          <t>Rozhovor</t>
         </is>
       </c>
       <c r="H23" s="5" t="n"/>
@@ -1355,78 +1559,90 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>#96</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>F-44</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>F-18</t>
+          <t>F-20</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Plán tréninku</t>
+          <t>Záznam tréninku</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Kopie plánu / šablona trenéra</t>
+          <t>Statistiky, videa na serveru a integrace</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Trenér zkopíruje osvědčený plán k dalšímu psovi.</t>
+          <t>Graf vývoje úspěšnosti, nahrávání videí na vlastní server a napojení na Stravu. Úspěch se v praxi číslem neměří (H5 podpořena) a vlastní úložiště videí je drahé.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Dávají trenéři podobné plány více klientům? (FB2, otázka 7)</t>
-        </is>
-      </c>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="n"/>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="n"/>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>F-27, F-28, F-29</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>F-19</t>
+          <t>F-21</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Týdenní rozvrh</t>
+          <t>Zpětná vazba</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Týdenní kalendář</t>
+          <t>Vlákno u tréninku</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Aktuální týden po dnech, tréninky všech psů najednou, barevně podle psa. Po kliknutí na den karta tréninku se seznamem cviků.</t>
+          <t>Psovod pošle s tréninkem komentář, trenér mu odpoví ve vlákně pod konkrétním tréninkem a reaguje na video. Vlákno unese dialog i doptávání (jak pes spal, jestli se chyba opakuje). Nahrazuje WhatsApp.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -1445,31 +1661,41 @@
           <t>Odsouhlaseno</t>
         </is>
       </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>F-30</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>F-20</t>
+          <t>F-22</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Týdenní rozvrh</t>
+          <t>Zpětná vazba</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Naplánování tréninku na den</t>
+          <t>Přehled klientů pro trenéra</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Tréninky se zařadí do dnů v týdnu a období (od–do). Rozvrh se zobrazuje v týdnech a dnech jako v aplikaci Runna.</t>
+          <t>Trenér vidí jen své klienty a jejich psy, plány a záznamy. Fronta „čeká na reakci“ mu ukáže dotazy a záznamy, na které ještě neodpověděl. Je to pomocník, ne kontrola plnění.</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Trenér, psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -1484,39 +1710,49 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Kdo zařazuje do dnů tréninky z cíle od trenéra, trenér, nebo psovod? (FB2, otázka 2). Svůj vlastní cíl si psovod naplánuje sám.</t>
+          <t>Potvrzeno (PO, FB1): přehled svěřenců odpovídá potřebě.</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>#81, #82, #83</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>F-31, F-32</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>F-21</t>
+          <t>F-23</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Týdenní rozvrh</t>
+          <t>Zpětná vazba</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Přesunout, nebo přeskočit trénink</t>
+          <t>Štítek „nová odpověď“</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Když trénink v daný den neproběhne, psovod ho jedním krokem přesune na jiný den či týden, nebo ho přeskočí, aby nevznikala lavina nedodělků (vzor Runna).</t>
+          <t>Psovod v Týdnu a u tréninku vidí, že mu trenér odpověděl; trenér vidí nové záznamy. Bez toho psovod odpověď nenajde.</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -1526,49 +1762,55 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>Co se stane s přeskočeným cvikem v plánu a vidí to trenér? (FB2, otázka 4)</t>
-        </is>
-      </c>
+          <t>Rozhovor</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="n"/>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>#84</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>F-33</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>F-22</t>
+          <t>F-24</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Týdenní rozvrh</t>
+          <t>Zpětná vazba</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Přepínání týdnů</t>
+          <t>E-mailová upozornění</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Zpět (co se odcvičilo) i dopředu (plánování).</t>
+          <t>Psovod nebo trenér dostane e-mail o nové odpovědi, záznamu nebo změně plánu.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -1576,131 +1818,153 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H28" s="5" t="n"/>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Stačí upozornění v aplikaci? (otázka 5)</t>
+        </is>
+      </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>#97</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>F-46</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>F-23</t>
+          <t>F-25</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Týdenní rozvrh</t>
+          <t>Tržiště a platby</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Zanedbané disciplíny</t>
+          <t>Tržiště plánů</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Upozornění, že některá disciplína tento týden nemá trénink. Neodcvičené tréninky řeší F-21.</t>
+          <t>Veřejné tržiště plánů z původního briefu.</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>Více disciplín trenérce práci navíc nedělá (H1 oslabena).</t>
-        </is>
-      </c>
+          <t>Klient</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="n"/>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="n"/>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>F-34</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>F-43</t>
+          <t>F-26</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Tržiště a platby</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Průchod tréninkem</t>
+          <t>Předplatné a platby</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Psovod otevře dnešní trénink a prochází cviky jeden po druhém („Aktuální cvik 3/20“), na konci přejde na obrazovku „Konec“.</t>
+          <t>Trenér platí za aktivního klienta: 3 zdarma, pak 49 Kč měsíčně za každého dalšího, strop 1 490 Kč měsíčně. Psovod 0 Kč. Tento semestr platby nestavíme.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Mimo rozsah</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Tým</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Šipky = další cvik v dnešním tréninku. Každý cvik ukazuje instrukci a kritérium (F-13).</t>
+          <t>Ceník je návrh týmu, viz lean-canvas.md (otázka 8).</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="n"/>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>F-35</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>F-24</t>
+          <t>F-27</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Technický základ</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Odeslání tréninku</t>
+          <t>Staging, CI/CD a zálohy</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Na obrazovce „Konec“ psovod zadá % úspěšnosti, rychlé hodnocení (soustředění, opakované chyby) a poznámku a odešle trénink trenérovi. Psovod bez trenéra si záznam uloží do deníku. Rychle, z mobilu.</t>
+          <t>Každá změna projde CI a po merge do main se nasadí na staging, kde ji PO uvidí dřív než uživatelé. Databáze se pravidelně zálohuje, aby historie tréninků nezmizela.</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -1710,134 +1974,156 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>Za cvik, nebo za celý trénink? Jak má psovod % určit? Trenérka měří úspěch kvalitativně (H5). (FB2, otázka 3)</t>
-        </is>
-      </c>
+          <t>Tým</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="n"/>
       <c r="I31" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>#86, #90</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>F-36, F-41</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>F-25</t>
+          <t>F-28</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Technický základ</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Video z tréninku</t>
+          <t>Monitoring a logy</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Na obrazovce „Konec“ psovod vloží odkaz na video z tréninku (YouTube unlisted, cloud), takže video už neleží odpojené v galerii.</t>
+          <t>O chybě se dozvíme dřív než uživatel.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Nice to have</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Jak klientům vložení odkazu usnadnit? (FB2, otázka 11)</t>
-        </is>
-      </c>
+          <t>Tým</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="n"/>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Odsouhlaseno</t>
+          <t>Navrženo</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>#98</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>F-42</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>F-44</t>
+          <t>F-29</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Technický základ</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Kontext k záznamu</t>
+          <t>Oprávnění a osobní údaje</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Psovod u záznamu volitelně vyplní okolnosti (jak pes spal, prostředí, jestli se chyba opakuje), na které se trenérka jinak doptává.</t>
+          <t>Psovod vidí jen své psy a záznamy, trenér jen psy, které s ním klient sdílí. Souhlas se zpracováním osobních údajů a smazání účtu včetně dat.</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Nice to have</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H33" s="5" t="n"/>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>#85, #88</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>F-38, F-39</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>F-26</t>
+          <t>F-30</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Technický základ</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Historie tréninků psa</t>
+          <t>Automatické testy</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Na detailu psa jsou „Aktivity“: odcvičené tréninky po dnech s videi a odpověďmi trenéra. Hodnota hlavně pro psovoda, který se k videím a zpětné vazbě vrací (trenérka ne).</t>
+          <t>Hlavní obrana proti chybám od agenta, hlavně v logice nelineárního plánu.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -1847,7 +2133,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="H34" s="5" t="n"/>
@@ -1856,83 +2142,103 @@
           <t>Navrženo</t>
         </is>
       </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>#87</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>F-37</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>F-27</t>
+          <t>F-31</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Technický základ</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Graf vývoje úspěšnosti</t>
+          <t>Odesílání e-mailů</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Vývoj % v čase u psa nebo plánu.</t>
+          <t>Aplikace posílá pozvánky klientům a obnovu hesla. Podle standupu 15. 10. mají e-maily fungovat už ve sprintu 2.</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Mimo rozsah</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Rozhovor</t>
+          <t>Klient</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>Úspěch se v praxi číslem neměří (H5 podpořena).</t>
+          <t>Jakou službu použít? Počítáme s bezplatným tarifem.</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Navrženo</t>
+          <t>Odsouhlaseno</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>#91</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>F-48</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>F-28</t>
+          <t>F-32</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Záznam tréninku</t>
+          <t>Technický základ</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Nahrávání videí na náš server</t>
+          <t>Použitelnost na mobilu</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Vlastní úložiště videí je drahé, v MVP ho nestavíme (viz F-25, otázka 6).</t>
+          <t>Psovod zapisuje venku po tréninku, aplikace musí fungovat na telefonu.</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Mimo rozsah</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -1940,724 +2246,202 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H36" s="5" t="n"/>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Rozhodnuto: responzivní webová aplikace.</t>
+        </is>
+      </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
           <t>Odsouhlaseno</t>
         </is>
       </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>#89</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>F-40</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>F-29</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Záznam tréninku</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Napojení na Stravu</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Import canicrossových běhů z běžeckých aplikací.</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Psovod</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>Mimo rozsah</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>Klient</t>
-        </is>
-      </c>
+      <c r="A37" s="5" t="n"/>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
       <c r="H37" s="5" t="n"/>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="I37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>F-30</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Zpětná vazba</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Komentáře k tréninku</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Psovod pošle s tréninkem komentář, trenér mu odpoví ve vlákně pod konkrétním tréninkem a reaguje na video. Vlákno unese dialog i doptávání (jak pes spal, jestli se chyba opakuje). Nahrazuje WhatsApp.</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Psovod, trenér</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>Klient</t>
-        </is>
-      </c>
+      <c r="A38" s="5" t="n"/>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="n"/>
       <c r="H38" s="5" t="n"/>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>Odsouhlaseno</t>
-        </is>
-      </c>
+      <c r="I38" s="5" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>F-31</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Zpětná vazba</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Seznam klientů</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Trenér vidí své klienty (jméno, e-mail) a přes ně jejich psy, plány a odcvičené tréninky.</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Trenér</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>Potvrzeno (PO, FB1): horní přehled svěřenců odpovídá pohledu trenéra.</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>Odsouhlaseno</t>
-        </is>
-      </c>
+      <c r="A39" s="5" t="n"/>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="5" t="n"/>
+      <c r="I39" s="5" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>F-32</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Zpětná vazba</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Čeká na reakci</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Fronta dotazů a záznamů od klientů, na které trenér ještě neodpověděl. Slouží jako pomocník, ne kontrola plnění: trenérka od klientů nic nevyžaduje a pokrok pozná na další lekci.</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Trenér</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>Rozhovor</t>
-        </is>
-      </c>
+      <c r="A40" s="5" t="n"/>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="5" t="n"/>
       <c r="H40" s="5" t="n"/>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="I40" s="5" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>F-33</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Zpětná vazba</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>Štítek „nová odpověď“</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Psovod v Týdnu a u tréninku vidí, že mu trenér odpověděl; trenér vidí nové záznamy. Bez toho psovod odpověď nenajde.</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Psovod, trenér</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>Rozhovor</t>
-        </is>
-      </c>
+      <c r="A41" s="5" t="n"/>
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="5" t="n"/>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="5" t="n"/>
       <c r="H41" s="5" t="n"/>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="I41" s="5" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>F-46</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Zpětná vazba</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>E-mailová upozornění</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Psovod nebo trenér dostane e-mail o nové odpovědi, záznamu nebo změně plánu.</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Psovod, trenér</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>Nice to have</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>Předpoklad týmu</t>
-        </is>
-      </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>Stačí upozornění v aplikaci, nebo je potřeba i e-mail? (FB2, otázka 5)</t>
-        </is>
-      </c>
-      <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="A42" s="5" t="n"/>
+      <c r="B42" s="5" t="n"/>
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="5" t="n"/>
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="5" t="n"/>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="5" t="n"/>
+      <c r="I42" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>F-34</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Tržiště a platby</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Prodej a nákup plánů, hodnocení</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Veřejné tržiště plánů z původního briefu.</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Psovod, trenér</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>Mimo rozsah</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>Klient</t>
-        </is>
-      </c>
+      <c r="A43" s="5" t="n"/>
+      <c r="B43" s="5" t="n"/>
+      <c r="C43" s="5" t="n"/>
+      <c r="D43" s="5" t="n"/>
+      <c r="E43" s="5" t="n"/>
+      <c r="F43" s="5" t="n"/>
+      <c r="G43" s="5" t="n"/>
       <c r="H43" s="5" t="n"/>
-      <c r="I43" s="5" t="inlineStr">
-        <is>
-          <t>Odsouhlaseno</t>
-        </is>
-      </c>
+      <c r="I43" s="5" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>F-35</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Tržiště a platby</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Předplatné a platby</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Trenér platí za aktivního klienta: 3 zdarma, pak 49 Kč měsíčně za každého dalšího, strop 1 490 Kč měsíčně. Psovod 0 Kč. Tento semestr platby nestavíme.</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Trenér</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>Mimo rozsah</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>Ceník je návrh týmu, viz lean-canvas.md a nakladova-struktura.xlsx (FB2, otázka 8).</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>Odsouhlaseno</t>
-        </is>
-      </c>
+      <c r="A44" s="5" t="n"/>
+      <c r="B44" s="5" t="n"/>
+      <c r="C44" s="5" t="n"/>
+      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="5" t="n"/>
+      <c r="G44" s="5" t="n"/>
+      <c r="H44" s="5" t="n"/>
+      <c r="I44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>F-36</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>Technický základ</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>Staging a CI/CD</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Každá změna se otestuje a nasadí na staging, kde ji PO uvidí dřív než uživatelé.</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="H45" s="5" t="inlineStr">
-        <is>
-          <t>Kdo bude mít přístup na staging?</t>
-        </is>
-      </c>
-      <c r="I45" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="A45" s="5" t="n"/>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="5" t="n"/>
+      <c r="I45" s="5" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>F-37</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Technický základ</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Automatické testy</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Hlavní obrana proti chybám od agenta, hlavně v logice nelineárního plánu.</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
+      <c r="A46" s="5" t="n"/>
+      <c r="B46" s="5" t="n"/>
+      <c r="C46" s="5" t="n"/>
+      <c r="D46" s="5" t="n"/>
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="5" t="n"/>
+      <c r="G46" s="5" t="n"/>
       <c r="H46" s="5" t="n"/>
-      <c r="I46" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="I46" s="5" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>F-38</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Technický základ</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Oprávnění</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Kdo vidí a upravuje psa, plán, záznamy a komentáře (psovod, trenér, cizí).</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
+      <c r="A47" s="5" t="n"/>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
       <c r="H47" s="5" t="n"/>
-      <c r="I47" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="I47" s="5" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>F-39</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Technický základ</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Osobní údaje a smazání účtu</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Souhlas se zpracováním, smazání účtu včetně dat.</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Psovod, trenér</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
+      <c r="A48" s="5" t="n"/>
+      <c r="B48" s="5" t="n"/>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="5" t="n"/>
+      <c r="F48" s="5" t="n"/>
+      <c r="G48" s="5" t="n"/>
       <c r="H48" s="5" t="n"/>
-      <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="I48" s="5" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>F-40</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Technický základ</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>Použitelnost na mobilu</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Psovod zapisuje venku po tréninku, aplikace musí fungovat na telefonu.</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Psovod, trenér</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>Klient</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>Rozhodnuto: responzivní webová aplikace (optimalizovaná pro mobil / PWA). Nativní aplikace v App Store / Google Play mimo rozsah pilotu.</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>Odsouhlaseno</t>
-        </is>
-      </c>
+      <c r="A49" s="5" t="n"/>
+      <c r="B49" s="5" t="n"/>
+      <c r="C49" s="5" t="n"/>
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="5" t="n"/>
+      <c r="F49" s="5" t="n"/>
+      <c r="G49" s="5" t="n"/>
+      <c r="H49" s="5" t="n"/>
+      <c r="I49" s="5" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>F-41</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Technický základ</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Zálohy dat</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Pravidelná záloha databáze, aby historie tréninků nezmizela.</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
+      <c r="A50" s="5" t="n"/>
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="5" t="n"/>
+      <c r="D50" s="5" t="n"/>
+      <c r="E50" s="5" t="n"/>
+      <c r="F50" s="5" t="n"/>
+      <c r="G50" s="5" t="n"/>
       <c r="H50" s="5" t="n"/>
-      <c r="I50" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="I50" s="5" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>F-42</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Technický základ</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>Monitoring a logy</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>O chybě se dozvíme dřív než uživatel.</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>Nice to have</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
+      <c r="A51" s="5" t="n"/>
+      <c r="B51" s="5" t="n"/>
+      <c r="C51" s="5" t="n"/>
+      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="5" t="n"/>
+      <c r="F51" s="5" t="n"/>
+      <c r="G51" s="5" t="n"/>
       <c r="H51" s="5" t="n"/>
-      <c r="I51" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="I51" s="5" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>F-48</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Technický základ</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>Odesílání e-mailů</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>Aplikace posílá e-maily: pozvánku klienta (F-08) a obnovu hesla (F-02). Klient je nevidí, ale bez nich tyto features nefungují.</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>MVP</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
-          <t>Tým</t>
-        </is>
-      </c>
-      <c r="H52" s="5" t="inlineStr">
-        <is>
-          <t>Jakou službu použít? Počítáme s bezplatným tarifem e-mailové služby, v cashflow proto bez nákladu.</t>
-        </is>
-      </c>
-      <c r="I52" s="5" t="inlineStr">
-        <is>
-          <t>Navrženo</t>
-        </is>
-      </c>
+      <c r="A52" s="5" t="n"/>
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="5" t="n"/>
+      <c r="D52" s="5" t="n"/>
+      <c r="E52" s="5" t="n"/>
+      <c r="F52" s="5" t="n"/>
+      <c r="G52" s="5" t="n"/>
+      <c r="H52" s="5" t="n"/>
+      <c r="I52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>

</xml_diff>